<commit_message>
Remove external temperature sensing and publish complete single-page Revision D schematic
Update the realistic README assembly illustration, schematic, netlist and shopping documents. Reserve fault 9 without renumbering stuck J, retain built-in driver thermal protection, and verify the temperature-branch-only wiring change. Local validation: 225 deterministic tests and schematic/export checks pass.
</commit_message>
<xml_diff>
--- a/docs/assets/procurement/shopping-list.xlsx
+++ b/docs/assets/procurement/shopping-list.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="Re13139757438462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rfb75f53389144b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="R6f9594dd227a46a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R8b7eb7b9503d4fdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -200,7 +200,7 @@
         <x:color rgb="FF805B15"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CA"/>
         </x:patternFill>
       </x:fill>
@@ -463,7 +463,7 @@
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Planning budget • 4 October 2026 • USD • not a delivered quotation</x:v>
+        <x:v>Revision D, 7 October 2026. Prices reviewed 4 October. USD planning budget.</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
@@ -495,7 +495,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>SUM(G20:G52)</x:f>
-        <x:v>624.36</x:v>
+        <x:v>609.6600000000001</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="18" t="str">
@@ -527,7 +527,7 @@
       </x:c>
       <x:c r="E7" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D7)</x:f>
-        <x:v>64.42</x:v>
+        <x:v>49.72</x:v>
       </x:c>
       <x:c r="F7" s="3"/>
       <x:c r="G7" s="3"/>
@@ -616,7 +616,7 @@
       </x:c>
       <x:c r="B11" s="9" t="n">
         <x:f>ROUND((SUM(B6:B8)-B9)*B10,2)</x:f>
-        <x:v>56.95</x:v>
+        <x:v>55.74</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3" t="str">
@@ -643,7 +643,7 @@
       </x:c>
       <x:c r="B12" s="10" t="n">
         <x:f>SUM(B6:B8)-B9+B11</x:f>
-        <x:v>747.3100000000001</x:v>
+        <x:v>731.4000000000001</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3" t="str">
@@ -681,7 +681,7 @@
       </x:c>
       <x:c r="B14" s="9" t="n">
         <x:f>SUMIFS(G20:G52,F20:F52,"Published")</x:f>
-        <x:v>285.37</x:v>
+        <x:v>270.6700000000001</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
@@ -1130,786 +1130,765 @@
       </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
-      <x:c r="A30" s="3" t="str">
-        <x:v>Control</x:v>
-      </x:c>
-      <x:c r="B30" s="3" t="str">
-        <x:v>Genuine DS18B20+ TO-92</x:v>
+      <x:c r="A30" s="22" t="str">
+        <x:v>Assembly</x:v>
+      </x:c>
+      <x:c r="B30" s="22" t="str">
+        <x:v>Exact resistors, diodes and capacitors</x:v>
       </x:c>
       <x:c r="C30" s="21" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D30" s="3" t="str">
-        <x:v>sensor</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D30" s="22" t="str">
+        <x:v>small lot</x:v>
       </x:c>
       <x:c r="E30" s="12" t="n">
-        <x:v>7.35</x:v>
-      </x:c>
-      <x:c r="F30" s="3" t="str">
-        <x:v>Published</x:v>
-      </x:c>
-      <x:c r="G30" s="9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F30" s="22" t="str">
+        <x:v>Allowance</x:v>
+      </x:c>
+      <x:c r="G30" s="23" t="n">
         <x:f>C30*E30</x:f>
-        <x:v>14.7</x:v>
-      </x:c>
-      <x:c r="H30" s="3" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H30" s="22" t="str">
+        <x:v>DigiKey / Mouser</x:v>
       </x:c>
       <x:c r="I30" s="3"/>
       <x:c r="J30" s="3" t="str">
-        <x:v>Powered three-wire mode; exterior sensor needs protected termination.</x:v>
+        <x:v>Full quantities and ratings are in shopping guide and Rev D BOM. Buy small spare quantities.</x:v>
       </x:c>
       <x:c r="K30" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/analog-devices-inc-maxim-integrated/DS18B20/956983</x:v>
+        <x:v>https://www.digikey.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
-      <x:c r="A31" s="22" t="str">
+      <x:c r="A31" s="3" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B31" s="22" t="str">
-        <x:v>Exact resistors, diodes and capacitors</x:v>
+      <x:c r="B31" s="3" t="str">
+        <x:v>FR4 perfboard, Nano headers and sockets</x:v>
       </x:c>
       <x:c r="C31" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D31" s="22" t="str">
-        <x:v>small lot</x:v>
+      <x:c r="D31" s="3" t="str">
+        <x:v>set</x:v>
       </x:c>
       <x:c r="E31" s="12" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F31" s="22" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F31" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G31" s="23" t="n">
+      <x:c r="G31" s="9" t="n">
         <x:f>C31*E31</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H31" s="22" t="str">
-        <x:v>DigiKey / Mouser</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H31" s="3" t="str">
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I31" s="3"/>
       <x:c r="J31" s="3" t="str">
-        <x:v>Full quantities and ratings are in shopping guide and Rev C BOM. Buy small spare quantities.</x:v>
+        <x:v>Soldered carrier with secure mounting; ordinary loose Dupont jumpers are for bench use only.</x:v>
       </x:c>
       <x:c r="K31" s="15" t="str">
-        <x:v>https://www.digikey.com/</x:v>
+        <x:v>https://www.amazon.com/s?k=FR4+perfboard+2.54mm+headers+female+socket</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
-      <x:c r="A32" s="3" t="str">
+      <x:c r="A32" s="22" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B32" s="3" t="str">
-        <x:v>FR4 perfboard, Nano headers and sockets</x:v>
+      <x:c r="B32" s="22" t="str">
+        <x:v>12 V, 5 V and ground distribution terminals</x:v>
       </x:c>
       <x:c r="C32" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D32" s="3" t="str">
+      <x:c r="D32" s="22" t="str">
         <x:v>set</x:v>
       </x:c>
       <x:c r="E32" s="12" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F32" s="3" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F32" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G32" s="9" t="n">
+      <x:c r="G32" s="23" t="n">
         <x:f>C32*E32</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H32" s="3" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H32" s="22" t="str">
         <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I32" s="3"/>
       <x:c r="J32" s="3" t="str">
-        <x:v>Soldered carrier with secure mounting; ordinary loose Dupont jumpers are for bench use only.</x:v>
+        <x:v>Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
       </x:c>
       <x:c r="K32" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=FR4+perfboard+2.54mm+headers+female+socket</x:v>
+        <x:v>https://www.amazon.com/s?k=covered+barrier+terminal+block+bus+bar</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
-      <x:c r="A33" s="22" t="str">
+      <x:c r="A33" s="3" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B33" s="22" t="str">
-        <x:v>12 V, 5 V and ground distribution terminals</x:v>
+      <x:c r="B33" s="3" t="str">
+        <x:v>Stranded copper internal hookup wire</x:v>
       </x:c>
       <x:c r="C33" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D33" s="22" t="str">
-        <x:v>set</x:v>
+      <x:c r="D33" s="3" t="str">
+        <x:v>assortment</x:v>
       </x:c>
       <x:c r="E33" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F33" s="22" t="str">
+      <x:c r="F33" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G33" s="23" t="n">
+      <x:c r="G33" s="9" t="n">
         <x:f>C33*E33</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="H33" s="22" t="str">
+      <x:c r="H33" s="3" t="str">
         <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I33" s="3"/>
       <x:c r="J33" s="3" t="str">
-        <x:v>Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
+        <x:v>22 AWG signal wire planning only; load/feed gauges subject to H2. Avoid copper-clad aluminum.</x:v>
       </x:c>
       <x:c r="K33" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=covered+barrier+terminal+block+bus+bar</x:v>
+        <x:v>https://www.amazon.com/s?k=stranded+copper+hookup+wire+22+awg+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
-      <x:c r="A34" s="3" t="str">
+      <x:c r="A34" s="22" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B34" s="3" t="str">
-        <x:v>Stranded copper internal hookup wire</x:v>
+      <x:c r="B34" s="22" t="str">
+        <x:v>Jacketed outdoor harness cable</x:v>
       </x:c>
       <x:c r="C34" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D34" s="3" t="str">
-        <x:v>assortment</x:v>
+      <x:c r="D34" s="22" t="str">
+        <x:v>length allowance</x:v>
       </x:c>
       <x:c r="E34" s="12" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F34" s="3" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F34" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G34" s="9" t="n">
+      <x:c r="G34" s="23" t="n">
         <x:f>C34*E34</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H34" s="3" t="str">
-        <x:v>Amazon</x:v>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H34" s="22" t="str">
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I34" s="3"/>
       <x:c r="J34" s="3" t="str">
-        <x:v>22 AWG signal wire planning only; load/feed gauges subject to H2. Avoid copper-clad aluminum.</x:v>
+        <x:v>Measure runs first. Lamp loom needs twenty color conductors plus suitably sized common return(s).</x:v>
       </x:c>
       <x:c r="K34" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=stranded+copper+hookup+wire+22+awg+kit</x:v>
+        <x:v>https://www.amazon.com/s?k=outdoor+multiconductor+copper+control+cable</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
-      <x:c r="A35" s="22" t="str">
+      <x:c r="A35" s="3" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B35" s="22" t="str">
-        <x:v>Jacketed outdoor harness cable</x:v>
+      <x:c r="B35" s="3" t="str">
+        <x:v>Locking sealed cable connectors</x:v>
       </x:c>
       <x:c r="C35" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D35" s="22" t="str">
-        <x:v>length allowance</x:v>
+      <x:c r="D35" s="3" t="str">
+        <x:v>set</x:v>
       </x:c>
       <x:c r="E35" s="12" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F35" s="22" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F35" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G35" s="23" t="n">
+      <x:c r="G35" s="9" t="n">
         <x:f>C35*E35</x:f>
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H35" s="22" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H35" s="3" t="str">
+        <x:v>Amazon / distributor</x:v>
       </x:c>
       <x:c r="I35" s="3"/>
       <x:c r="J35" s="3" t="str">
-        <x:v>Measure runs first. Lamp loom needs twenty color conductors plus suitably sized common return(s).</x:v>
+        <x:v>Use genuine rated parts with matching wire seals. Reused 14-pin machine connector excluded.</x:v>
       </x:c>
       <x:c r="K35" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=outdoor+multiconductor+copper+control+cable</x:v>
+        <x:v>https://www.amazon.com/s?k=Deutsch+DT+sealed+connector+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
-      <x:c r="A36" s="3" t="str">
+      <x:c r="A36" s="22" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B36" s="3" t="str">
-        <x:v>Locking sealed cable connectors</x:v>
+      <x:c r="B36" s="22" t="str">
+        <x:v>Heat shrink, ferrules, loom and labels</x:v>
       </x:c>
       <x:c r="C36" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D36" s="3" t="str">
-        <x:v>set</x:v>
+      <x:c r="D36" s="22" t="str">
+        <x:v>small lot</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F36" s="3" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F36" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G36" s="9" t="n">
+      <x:c r="G36" s="23" t="n">
         <x:f>C36*E36</x:f>
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="H36" s="3" t="str">
-        <x:v>Amazon / distributor</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H36" s="22" t="str">
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I36" s="3"/>
       <x:c r="J36" s="3" t="str">
-        <x:v>Use genuine rated parts with matching wire seals. Reused 14-pin machine connector excluded.</x:v>
+        <x:v>Adhesive-lined shrink at splices; secure cable strain relief. Reduce if already owned.</x:v>
       </x:c>
       <x:c r="K36" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=Deutsch+DT+sealed+connector+kit</x:v>
+        <x:v>https://www.amazon.com/s?k=adhesive+lined+heat+shrink+ferrules+wire+labels</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
-      <x:c r="A37" s="22" t="str">
+      <x:c r="A37" s="3" t="str">
         <x:v>Assembly</x:v>
       </x:c>
-      <x:c r="B37" s="22" t="str">
-        <x:v>Heat shrink, ferrules, loom and labels</x:v>
+      <x:c r="B37" s="3" t="str">
+        <x:v>Standoffs, fasteners and mounting brackets</x:v>
       </x:c>
       <x:c r="C37" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D37" s="22" t="str">
+      <x:c r="D37" s="3" t="str">
         <x:v>small lot</x:v>
       </x:c>
       <x:c r="E37" s="12" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F37" s="22" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G37" s="23" t="n">
+      <x:c r="G37" s="9" t="n">
         <x:f>C37*E37</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H37" s="22" t="str">
-        <x:v>Amazon</x:v>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H37" s="3" t="str">
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I37" s="3"/>
       <x:c r="J37" s="3" t="str">
-        <x:v>Adhesive-lined shrink at splices; secure cable strain relief. Reduce if already owned.</x:v>
+        <x:v>Insulated board clearance above steel plate; mounting should not puncture the sealing cavity.</x:v>
       </x:c>
       <x:c r="K37" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=adhesive+lined+heat+shrink+ferrules+wire+labels</x:v>
+        <x:v>https://www.amazon.com/s?k=nylon+pcb+standoff+M3+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
-      <x:c r="A38" s="3" t="str">
-        <x:v>Assembly</x:v>
-      </x:c>
-      <x:c r="B38" s="3" t="str">
-        <x:v>Standoffs, fasteners and mounting brackets</x:v>
+      <x:c r="A38" s="22" t="str">
+        <x:v>Enclosure</x:v>
+      </x:c>
+      <x:c r="B38" s="22" t="str">
+        <x:v>Hammond 1554VA2GY opaque polycarbonate</x:v>
       </x:c>
       <x:c r="C38" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D38" s="3" t="str">
-        <x:v>small lot</x:v>
+      <x:c r="D38" s="22" t="str">
+        <x:v>box</x:v>
       </x:c>
       <x:c r="E38" s="12" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F38" s="3" t="str">
-        <x:v>Allowance</x:v>
-      </x:c>
-      <x:c r="G38" s="9" t="n">
+        <x:v>43.5</x:v>
+      </x:c>
+      <x:c r="F38" s="22" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G38" s="23" t="n">
         <x:f>C38*E38</x:f>
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H38" s="3" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>43.5</x:v>
+      </x:c>
+      <x:c r="H38" s="22" t="str">
+        <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I38" s="3"/>
       <x:c r="J38" s="3" t="str">
-        <x:v>Insulated board clearance above steel plate; mounting should not puncture the sealing cavity.</x:v>
+        <x:v>Nominal 240 x 160 x 90 mm. Preferred planning size; confirm physical layout before drilling.</x:v>
       </x:c>
       <x:c r="K38" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=nylon+pcb+standoff+M3+kit</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/miniature_cases/1554va2gy</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
-      <x:c r="A39" s="22" t="str">
+      <x:c r="A39" s="3" t="str">
         <x:v>Enclosure</x:v>
       </x:c>
-      <x:c r="B39" s="22" t="str">
-        <x:v>Hammond 1554VA2GY opaque polycarbonate</x:v>
+      <x:c r="B39" s="3" t="str">
+        <x:v>Hammond 1554VAPL mounting plate</x:v>
       </x:c>
       <x:c r="C39" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D39" s="22" t="str">
-        <x:v>box</x:v>
+      <x:c r="D39" s="3" t="str">
+        <x:v>plate</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
-        <x:v>43.5</x:v>
-      </x:c>
-      <x:c r="F39" s="22" t="str">
+        <x:v>9.25</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
         <x:v>Published</x:v>
       </x:c>
-      <x:c r="G39" s="23" t="n">
+      <x:c r="G39" s="9" t="n">
         <x:f>C39*E39</x:f>
-        <x:v>43.5</x:v>
-      </x:c>
-      <x:c r="H39" s="22" t="str">
+        <x:v>9.25</x:v>
+      </x:c>
+      <x:c r="H39" s="3" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I39" s="3"/>
       <x:c r="J39" s="3" t="str">
-        <x:v>Nominal 240 x 160 x 90 mm. Preferred planning size; confirm physical layout before drilling.</x:v>
+        <x:v>Box plus plate clears advertised $49 free-shipping threshold; checkout confirmation still required.</x:v>
       </x:c>
       <x:c r="K39" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/miniature_cases/1554va2gy</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/subpanels/1554vapl</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
-      <x:c r="A40" s="3" t="str">
+      <x:c r="A40" s="22" t="str">
         <x:v>Enclosure</x:v>
       </x:c>
-      <x:c r="B40" s="3" t="str">
-        <x:v>Hammond 1554VAPL mounting plate</x:v>
+      <x:c r="B40" s="22" t="str">
+        <x:v>Bimed BM-ENX-2S-W cable glands</x:v>
       </x:c>
       <x:c r="C40" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D40" s="3" t="str">
-        <x:v>plate</x:v>
+      <x:c r="D40" s="22" t="str">
+        <x:v>5-pack</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
-        <x:v>9.25</x:v>
-      </x:c>
-      <x:c r="F40" s="3" t="str">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="F40" s="22" t="str">
         <x:v>Published</x:v>
       </x:c>
-      <x:c r="G40" s="9" t="n">
+      <x:c r="G40" s="23" t="n">
         <x:f>C40*E40</x:f>
-        <x:v>9.25</x:v>
-      </x:c>
-      <x:c r="H40" s="3" t="str">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="H40" s="22" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I40" s="3"/>
       <x:c r="J40" s="3" t="str">
-        <x:v>Box plus plate clears advertised $49 free-shipping threshold; checkout confirmation still required.</x:v>
+        <x:v>M12 x 1.5; jacket OD 3–6.5 mm. Use only where cable diameter fits; mounting hardware included.</x:v>
       </x:c>
       <x:c r="K40" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/subpanels/1554vapl</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/wire_-a-_cable_management/cable_glands/metric_thread/bm-enx-2s-w</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
-      <x:c r="A41" s="22" t="str">
+      <x:c r="A41" s="3" t="str">
         <x:v>Enclosure</x:v>
       </x:c>
-      <x:c r="B41" s="22" t="str">
-        <x:v>Bimed BM-ENX-2S-W cable glands</x:v>
+      <x:c r="B41" s="3" t="str">
+        <x:v>Larger glands, sealing plugs and seals</x:v>
       </x:c>
       <x:c r="C41" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D41" s="22" t="str">
-        <x:v>5-pack</x:v>
+      <x:c r="D41" s="3" t="str">
+        <x:v>allowance</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
-        <x:v>3.25</x:v>
-      </x:c>
-      <x:c r="F41" s="22" t="str">
-        <x:v>Published</x:v>
-      </x:c>
-      <x:c r="G41" s="23" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F41" s="3" t="str">
+        <x:v>Allowance</x:v>
+      </x:c>
+      <x:c r="G41" s="9" t="n">
         <x:f>C41*E41</x:f>
-        <x:v>3.25</x:v>
-      </x:c>
-      <x:c r="H41" s="22" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H41" s="3" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I41" s="3"/>
       <x:c r="J41" s="3" t="str">
-        <x:v>M12 x 1.5; jacket OD 3–6.5 mm. Use only where cable diameter fits; mounting hardware included.</x:v>
+        <x:v>Machine/display cable may need larger glands or matched multi-hole inserts; measure first.</x:v>
       </x:c>
       <x:c r="K41" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/wire_-a-_cable_management/cable_glands/metric_thread/bm-enx-2s-w</x:v>
+        <x:v>https://www.automationdirect.com/adc/overview/catalog/wire_-a-_cable_management/cable_glands</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
-      <x:c r="A42" s="3" t="str">
+      <x:c r="A42" s="22" t="str">
         <x:v>Enclosure</x:v>
       </x:c>
-      <x:c r="B42" s="3" t="str">
-        <x:v>Larger glands, sealing plugs and seals</x:v>
+      <x:c r="B42" s="22" t="str">
+        <x:v>Ten-lamp rail / rear wiring cover</x:v>
       </x:c>
       <x:c r="C42" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D42" s="3" t="str">
-        <x:v>allowance</x:v>
+      <x:c r="D42" s="22" t="str">
+        <x:v>assembly allowance</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F42" s="3" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F42" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G42" s="9" t="n">
+      <x:c r="G42" s="23" t="n">
         <x:f>C42*E42</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H42" s="3" t="str">
-        <x:v>AutomationDirect</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H42" s="22" t="str">
+        <x:v>Local / Amazon</x:v>
       </x:c>
       <x:c r="I42" s="3"/>
       <x:c r="J42" s="3" t="str">
-        <x:v>Machine/display cable may need larger glands or matched multi-hole inserts; measure first.</x:v>
+        <x:v>Plan approximately 300 mm long; verify actual grommet diameter/pitch. No rated finished housing selected.</x:v>
       </x:c>
       <x:c r="K42" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/overview/catalog/wire_-a-_cable_management/cable_glands</x:v>
+        <x:v>https://www.amazon.com/s?k=aluminum+u+channel+12+inch</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
-      <x:c r="A43" s="22" t="str">
+      <x:c r="A43" s="3" t="str">
         <x:v>Enclosure</x:v>
       </x:c>
-      <x:c r="B43" s="22" t="str">
-        <x:v>Ten-lamp rail / rear wiring cover</x:v>
+      <x:c r="B43" s="3" t="str">
+        <x:v>Meter electronics protection</x:v>
       </x:c>
       <x:c r="C43" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D43" s="22" t="str">
+      <x:c r="D43" s="3" t="str">
         <x:v>assembly allowance</x:v>
       </x:c>
       <x:c r="E43" s="12" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F43" s="22" t="str">
+      <x:c r="F43" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G43" s="23" t="n">
+      <x:c r="G43" s="9" t="n">
         <x:f>C43*E43</x:f>
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H43" s="22" t="str">
-        <x:v>Local / Amazon</x:v>
+      <x:c r="H43" s="3" t="str">
+        <x:v>Local / distributor</x:v>
       </x:c>
       <x:c r="I43" s="3"/>
       <x:c r="J43" s="3" t="str">
-        <x:v>Plan approximately 300 mm long; verify actual grommet diameter/pitch. No rated finished housing selected.</x:v>
+        <x:v>Dedicated splash/impact protection, supported plumbing and sealed terminations; exact housing pending geometry.</x:v>
       </x:c>
       <x:c r="K43" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=aluminum+u+channel+12+inch</x:v>
+        <x:v>https://www.polycase.com/wp-series</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
-      <x:c r="A44" s="3" t="str">
-        <x:v>Enclosure</x:v>
-      </x:c>
-      <x:c r="B44" s="3" t="str">
-        <x:v>Meter and exterior sensor protection</x:v>
+      <x:c r="A44" s="22" t="str">
+        <x:v>Water</x:v>
+      </x:c>
+      <x:c r="B44" s="22" t="str">
+        <x:v>Manual shutoff and cleanable inlet strainer</x:v>
       </x:c>
       <x:c r="C44" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D44" s="3" t="str">
-        <x:v>assembly allowance</x:v>
+      <x:c r="D44" s="22" t="str">
+        <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F44" s="3" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F44" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G44" s="9" t="n">
+      <x:c r="G44" s="23" t="n">
         <x:f>C44*E44</x:f>
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H44" s="3" t="str">
-        <x:v>Local / distributor</x:v>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H44" s="22" t="str">
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I44" s="3"/>
       <x:c r="J44" s="3" t="str">
-        <x:v>Dedicated splash/impact protection, supported plumbing and sealed terminations; exact housing pending geometry.</x:v>
+        <x:v>Reuse existing suitable items; select pressure rating and mesh for nozzle/meter requirements.</x:v>
       </x:c>
       <x:c r="K44" s="15" t="str">
-        <x:v>https://www.polycase.com/wp-series</x:v>
+        <x:v>https://www.amazon.com/s?k=garden+hose+shut+off+valve+inline+filter+brass</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
-      <x:c r="A45" s="22" t="str">
+      <x:c r="A45" s="3" t="str">
         <x:v>Water</x:v>
       </x:c>
-      <x:c r="B45" s="22" t="str">
-        <x:v>Manual shutoff and cleanable inlet strainer</x:v>
+      <x:c r="B45" s="3" t="str">
+        <x:v>Correct NPS meter adapters and seals</x:v>
       </x:c>
       <x:c r="C45" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D45" s="22" t="str">
-        <x:v>set allowance</x:v>
+      <x:c r="D45" s="3" t="str">
+        <x:v>pair allowance</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="F45" s="22" t="str">
+      <x:c r="F45" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G45" s="23" t="n">
+      <x:c r="G45" s="9" t="n">
         <x:f>C45*E45</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="H45" s="22" t="str">
-        <x:v>Amazon / local</x:v>
+      <x:c r="H45" s="3" t="str">
+        <x:v>Plumbing supplier</x:v>
       </x:c>
       <x:c r="I45" s="3"/>
       <x:c r="J45" s="3" t="str">
-        <x:v>Reuse existing suitable items; select pressure rating and mesh for nozzle/meter requirements.</x:v>
+        <x:v>PROCUREMENT HOLD: straight NPS thread and actual seal geometry must match; NPT or cone-seat swivel is not assumed compatible.</x:v>
       </x:c>
       <x:c r="K45" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=garden+hose+shut+off+valve+inline+filter+brass</x:v>
+        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
-      <x:c r="A46" s="3" t="str">
+      <x:c r="A46" s="22" t="str">
         <x:v>Water</x:v>
       </x:c>
-      <x:c r="B46" s="3" t="str">
-        <x:v>Correct NPS meter adapters and seals</x:v>
+      <x:c r="B46" s="22" t="str">
+        <x:v>Garden-hose to valve NPT fittings</x:v>
       </x:c>
       <x:c r="C46" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D46" s="3" t="str">
-        <x:v>pair allowance</x:v>
+      <x:c r="D46" s="22" t="str">
+        <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F46" s="3" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F46" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G46" s="9" t="n">
+      <x:c r="G46" s="23" t="n">
         <x:f>C46*E46</x:f>
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H46" s="3" t="str">
-        <x:v>Plumbing supplier</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H46" s="22" t="str">
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I46" s="3"/>
       <x:c r="J46" s="3" t="str">
-        <x:v>PROCUREMENT HOLD: straight NPS thread and actual seal geometry must match; NPT or cone-seat swivel is not assumed compatible.</x:v>
+        <x:v>US garden hose thread is 3/4 GHT, distinct from 1/2 NPT valve threads. Include removable unions as required.</x:v>
       </x:c>
       <x:c r="K46" s="15" t="str">
-        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
+        <x:v>https://www.amazon.com/s?k=3%2F4+GHT+to+1%2F2+NPT+brass+adapter</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
-      <x:c r="A47" s="22" t="str">
+      <x:c r="A47" s="3" t="str">
         <x:v>Water</x:v>
       </x:c>
-      <x:c r="B47" s="22" t="str">
-        <x:v>Garden-hose to valve NPT fittings</x:v>
+      <x:c r="B47" s="3" t="str">
+        <x:v>Straight pipe, washers, supports and sealant</x:v>
       </x:c>
       <x:c r="C47" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D47" s="22" t="str">
-        <x:v>set allowance</x:v>
+      <x:c r="D47" s="3" t="str">
+        <x:v>small lot</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F47" s="22" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F47" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G47" s="23" t="n">
+      <x:c r="G47" s="9" t="n">
         <x:f>C47*E47</x:f>
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H47" s="22" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H47" s="3" t="str">
+        <x:v>Local</x:v>
       </x:c>
       <x:c r="I47" s="3"/>
       <x:c r="J47" s="3" t="str">
-        <x:v>US garden hose thread is 3/4 GHT, distinct from 1/2 NPT valve threads. Include removable unions as required.</x:v>
+        <x:v>Respect meter straight lengths and seal type. Do not seal NPS solely with PTFE tape.</x:v>
       </x:c>
       <x:c r="K47" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=3%2F4+GHT+to+1%2F2+NPT+brass+adapter</x:v>
+        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
-      <x:c r="A48" s="3" t="str">
-        <x:v>Water</x:v>
-      </x:c>
-      <x:c r="B48" s="3" t="str">
-        <x:v>Straight pipe, washers, supports and sealant</x:v>
+      <x:c r="A48" s="22" t="str">
+        <x:v>Enclosure</x:v>
+      </x:c>
+      <x:c r="B48" s="22" t="str">
+        <x:v>MG Chemicals 422C coating, small bottle</x:v>
       </x:c>
       <x:c r="C48" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D48" s="3" t="str">
-        <x:v>small lot</x:v>
+      <x:c r="D48" s="22" t="str">
+        <x:v>bottle allowance</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="F48" s="3" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F48" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G48" s="9" t="n">
+      <x:c r="G48" s="23" t="n">
         <x:f>C48*E48</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H48" s="3" t="str">
-        <x:v>Local</x:v>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H48" s="22" t="str">
+        <x:v>Amazon / distributor</x:v>
       </x:c>
       <x:c r="I48" s="3"/>
       <x:c r="J48" s="3" t="str">
-        <x:v>Respect meter straight lengths and seal type. Do not seal NPS solely with PTFE tape.</x:v>
+        <x:v>Later, after testing; mask contacts, connectors and vents. Not a substitute for the gasketed box.</x:v>
       </x:c>
       <x:c r="K48" s="15" t="str">
-        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
+        <x:v>https://www.amazon.com/s?k=MG+Chemicals+422C+55ml</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
-      <x:c r="A49" s="22" t="str">
-        <x:v>Enclosure</x:v>
-      </x:c>
-      <x:c r="B49" s="22" t="str">
-        <x:v>MG Chemicals 422C coating, small bottle</x:v>
+      <x:c r="A49" s="3" t="str">
+        <x:v>Bench</x:v>
+      </x:c>
+      <x:c r="B49" s="3" t="str">
+        <x:v>Temporary fused battery lead and small fuses</x:v>
       </x:c>
       <x:c r="C49" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D49" s="22" t="str">
-        <x:v>bottle allowance</x:v>
+      <x:c r="D49" s="3" t="str">
+        <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E49" s="12" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F49" s="22" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F49" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G49" s="23" t="n">
+      <x:c r="G49" s="9" t="n">
         <x:f>C49*E49</x:f>
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H49" s="22" t="str">
-        <x:v>Amazon / distributor</x:v>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H49" s="3" t="str">
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I49" s="3"/>
       <x:c r="J49" s="3" t="str">
-        <x:v>Later, after testing; mask contacts, connectors and vents. Not a substitute for the gasketed box.</x:v>
+        <x:v>Bench only, close to battery; size fuse to test stage and weakest wire. Not a new machine fuse block.</x:v>
       </x:c>
       <x:c r="K49" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=MG+Chemicals+422C+55ml</x:v>
+        <x:v>https://www.amazon.com/s?k=inline+ATO+fuse+holder+1A+2A+fuse</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
-      <x:c r="A50" s="3" t="str">
+      <x:c r="A50" s="22" t="str">
         <x:v>Bench</x:v>
       </x:c>
-      <x:c r="B50" s="3" t="str">
-        <x:v>Temporary fused battery lead and small fuses</x:v>
+      <x:c r="B50" s="22" t="str">
+        <x:v>250-ohm 0.1% 0.5 W removable test resistor</x:v>
       </x:c>
       <x:c r="C50" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D50" s="3" t="str">
-        <x:v>set allowance</x:v>
+      <x:c r="D50" s="22" t="str">
+        <x:v>resistor allowance</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F50" s="3" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F50" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G50" s="9" t="n">
+      <x:c r="G50" s="23" t="n">
         <x:f>C50*E50</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H50" s="3" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H50" s="22" t="str">
+        <x:v>DigiKey / Mouser</x:v>
       </x:c>
       <x:c r="I50" s="3"/>
       <x:c r="J50" s="3" t="str">
-        <x:v>Bench only, close to battery; size fuse to test stage and weakest wire. Not a new machine fuse block.</x:v>
+        <x:v>DAC test load only. Expected 1/3/5 V at 4/12/20 mA; remove before valve wiring.</x:v>
       </x:c>
       <x:c r="K50" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=inline+ATO+fuse+holder+1A+2A+fuse</x:v>
+        <x:v>https://www.digikey.com/en/products?keywords=250%20ohm%200.1%25%200.5W%20resistor</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
-      <x:c r="A51" s="22" t="str">
+      <x:c r="A51" s="3" t="str">
         <x:v>Bench</x:v>
       </x:c>
-      <x:c r="B51" s="22" t="str">
-        <x:v>250-ohm 0.1% 0.5 W removable test resistor</x:v>
+      <x:c r="B51" s="3" t="str">
+        <x:v>Micro-USB data cable</x:v>
       </x:c>
       <x:c r="C51" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D51" s="22" t="str">
-        <x:v>resistor allowance</x:v>
+      <x:c r="D51" s="3" t="str">
+        <x:v>cable allowance</x:v>
       </x:c>
       <x:c r="E51" s="12" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F51" s="22" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F51" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
-      <x:c r="G51" s="23" t="n">
+      <x:c r="G51" s="9" t="n">
         <x:f>C51*E51</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H51" s="22" t="str">
-        <x:v>DigiKey / Mouser</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H51" s="3" t="str">
+        <x:v>Amazon / existing</x:v>
       </x:c>
       <x:c r="I51" s="3"/>
       <x:c r="J51" s="3" t="str">
-        <x:v>DAC test load only. Expected 1/3/5 V at 4/12/20 mA; remove before valve wiring.</x:v>
+        <x:v>Set quantity to zero if owned. Must carry data, not charging-only.</x:v>
       </x:c>
       <x:c r="K51" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products?keywords=250%20ohm%200.1%25%200.5W%20resistor</x:v>
+        <x:v>https://www.amazon.com/s?k=micro+usb+data+cable</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
-      <x:c r="A52" s="3" t="str">
-        <x:v>Bench</x:v>
-      </x:c>
-      <x:c r="B52" s="3" t="str">
-        <x:v>Micro-USB data cable</x:v>
-      </x:c>
-      <x:c r="C52" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D52" s="3" t="str">
-        <x:v>cable allowance</x:v>
-      </x:c>
-      <x:c r="E52" s="12" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F52" s="3" t="str">
-        <x:v>Allowance</x:v>
-      </x:c>
-      <x:c r="G52" s="9" t="n">
-        <x:f>C52*E52</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H52" s="3" t="str">
-        <x:v>Amazon / existing</x:v>
-      </x:c>
+      <x:c r="A52" s="3"/>
+      <x:c r="B52" s="3"/>
+      <x:c r="C52" s="21"/>
+      <x:c r="D52" s="3"/>
+      <x:c r="E52" s="12"/>
+      <x:c r="F52" s="3"/>
+      <x:c r="G52" s="9"/>
+      <x:c r="H52" s="3"/>
       <x:c r="I52" s="3"/>
-      <x:c r="J52" s="3" t="str">
-        <x:v>Set quantity to zero if owned. Must carry data, not charging-only.</x:v>
-      </x:c>
-      <x:c r="K52" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=micro+usb+data+cable</x:v>
-      </x:c>
+      <x:c r="J52" s="3"/>
+      <x:c r="K52" s="15"/>
     </x:row>
     <x:row r="53" ht="26" customHeight="1">
       <x:c r="A53" s="3"/>

</xml_diff>

<commit_message>
Draw continuous overall wiring and refresh component purchasing list
</commit_message>
<xml_diff>
--- a/docs/assets/procurement/shopping-list.xlsx
+++ b/docs/assets/procurement/shopping-list.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="R6f9594dd227a46a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R8b7eb7b9503d4fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="R01d9dcc738004bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rcedf89cffe184b1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +14,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="$#,##0.00;[Red]($#,##0.00);$0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.00%"/>
+    <x:numFmt numFmtId="202" formatCode="$0.000"/>
+    <x:numFmt numFmtId="203" formatCode="0"/>
+    <x:numFmt numFmtId="204" formatCode="$0.00"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +70,13 @@
       <x:color rgb="FF637381"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF193348"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,6 +96,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F6F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F5"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -121,7 +139,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -188,6 +206,45 @@
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -463,7 +520,7 @@
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Revision D, 7 October 2026. Prices reviewed 4 October. USD planning budget.</x:v>
+        <x:v>Revision D · prices reviewed 7 October 2026 · USD planning budget; no temperature probes.</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
@@ -495,7 +552,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>SUM(G20:G52)</x:f>
-        <x:v>609.6600000000001</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="18" t="str">
@@ -519,7 +576,7 @@
       </x:c>
       <x:c r="B7" s="9" t="n">
         <x:f>SUM(E57:E62)</x:f>
-        <x:v>46</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3" t="str">
@@ -527,7 +584,7 @@
       </x:c>
       <x:c r="E7" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D7)</x:f>
-        <x:v>49.72</x:v>
+        <x:v>49.239999999999995</x:v>
       </x:c>
       <x:c r="F7" s="3"/>
       <x:c r="G7" s="3"/>
@@ -597,7 +654,7 @@
       </x:c>
       <x:c r="E10" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D10)</x:f>
-        <x:v>85</x:v>
+        <x:v>87.46000000000001</x:v>
       </x:c>
       <x:c r="F10" s="3"/>
       <x:c r="G10" s="3"/>
@@ -616,7 +673,7 @@
       </x:c>
       <x:c r="B11" s="9" t="n">
         <x:f>ROUND((SUM(B6:B8)-B9)*B10,2)</x:f>
-        <x:v>55.74</x:v>
+        <x:v>56.84</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3" t="str">
@@ -643,7 +700,7 @@
       </x:c>
       <x:c r="B12" s="10" t="n">
         <x:f>SUM(B6:B8)-B9+B11</x:f>
-        <x:v>731.4000000000001</x:v>
+        <x:v>745.84</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3" t="str">
@@ -651,7 +708,7 @@
       </x:c>
       <x:c r="E12" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D12)</x:f>
-        <x:v>17</x:v>
+        <x:v>18.36</x:v>
       </x:c>
       <x:c r="F12" s="3"/>
       <x:c r="G12" s="3"/>
@@ -681,7 +738,7 @@
       </x:c>
       <x:c r="B14" s="9" t="n">
         <x:f>SUMIFS(G20:G52,F20:F52,"Published")</x:f>
-        <x:v>270.6700000000001</x:v>
+        <x:v>312.00000000000006</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
@@ -701,7 +758,7 @@
       </x:c>
       <x:c r="B15" s="9" t="n">
         <x:f>SUMIFS(G20:G52,F20:F52,"Allowance")</x:f>
-        <x:v>338.99</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="C15" s="3"/>
       <x:c r="D15" s="3"/>
@@ -815,9 +872,9 @@
       <x:c r="H20" s="3" t="str">
         <x:v>SparkFun</x:v>
       </x:c>
-      <x:c r="I20" s="3"/>
-      <x:c r="J20" s="3" t="str">
-        <x:v>Combine with opto boards; Arduino direct is $12.90 before separate shipping. Headers required.</x:v>
+      <x:c r="I20" s="3" t="str"/>
+      <x:c r="J20" s="24" t="str">
+        <x:v>Refs: U1. Combine with opto boards; Arduino direct is $12.90 before separate shipping. Headers required.</x:v>
       </x:c>
       <x:c r="K20" s="15" t="str">
         <x:v>https://www.sparkfun.com/arduino-nano-every.html</x:v>
@@ -849,9 +906,9 @@
       <x:c r="H21" s="22" t="str">
         <x:v>U.S. Solid</x:v>
       </x:c>
-      <x:c r="I21" s="3"/>
-      <x:c r="J21" s="3" t="str">
-        <x:v>1/2-inch stainless; 9–24 V; five-wire 4–20 mA command and feedback. H4 qualification pending.</x:v>
+      <x:c r="I21" s="3" t="str"/>
+      <x:c r="J21" s="24" t="str">
+        <x:v>Refs: V1. 1/2-inch stainless; 9–24 V; five-wire 4–20 mA command and feedback. H4 qualification pending.</x:v>
       </x:c>
       <x:c r="K21" s="15" t="str">
         <x:v>https://ussolid.com/products/1-2-proportional-motorized-ball-valve-stainless-steel-dc-9-24v-4-20ma-control-5-wire-ip67-full-port</x:v>
@@ -883,9 +940,9 @@
       <x:c r="H22" s="3" t="str">
         <x:v>DFRobot</x:v>
       </x:c>
-      <x:c r="I22" s="3"/>
-      <x:c r="J22" s="3" t="str">
-        <x:v>3.3–5 V supply; keep exact SKU. Direct shipping resumes Oct 8.</x:v>
+      <x:c r="I22" s="3" t="str"/>
+      <x:c r="J22" s="24" t="str">
+        <x:v>Refs: U2. 3.3–5 V supply; keep exact SKU. Direct shipping resumes Oct 8.</x:v>
       </x:c>
       <x:c r="K22" s="15" t="str">
         <x:v>https://www.dfrobot.com/product-3073.html</x:v>
@@ -917,9 +974,9 @@
       <x:c r="H23" s="22" t="str">
         <x:v>DFRobot</x:v>
       </x:c>
-      <x:c r="I23" s="3"/>
-      <x:c r="J23" s="3" t="str">
-        <x:v>120-ohm receiver; analog output. Do not add a 250-ohm shunt in parallel.</x:v>
+      <x:c r="I23" s="3" t="str"/>
+      <x:c r="J23" s="24" t="str">
+        <x:v>Refs: U3. 120-ohm receiver; analog output. Do not add a 250-ohm shunt in parallel.</x:v>
       </x:c>
       <x:c r="K23" s="15" t="str">
         <x:v>https://www.dfrobot.com/product-1755.html</x:v>
@@ -951,9 +1008,9 @@
       <x:c r="H24" s="3" t="str">
         <x:v>SparkFun</x:v>
       </x:c>
-      <x:c r="I24" s="3"/>
-      <x:c r="J24" s="3" t="str">
-        <x:v>Three channels used; external input resistors/diodes still required.</x:v>
+      <x:c r="I24" s="3" t="str"/>
+      <x:c r="J24" s="24" t="str">
+        <x:v>Refs: O1, O2. Three channels used; external input resistors/diodes still required.</x:v>
       </x:c>
       <x:c r="K24" s="15" t="str">
         <x:v>https://www.sparkfun.com/sparkfun-opto-isolator-breakout.html</x:v>
@@ -985,9 +1042,9 @@
       <x:c r="H25" s="22" t="str">
         <x:v>Serial Wombat</x:v>
       </x:c>
-      <x:c r="I25" s="3"/>
-      <x:c r="J25" s="3" t="str">
-        <x:v>PRICE/STOCK UNVERIFIED. $30 each is a budgeting placeholder, not a quotation. Procurement hold.</x:v>
+      <x:c r="I25" s="3" t="str"/>
+      <x:c r="J25" s="24" t="str">
+        <x:v>Refs: HSD1, HSD2, HSD3. PRICE/STOCK UNVERIFIED. $30 each is a budgeting placeholder, not a quotation. Procurement hold.</x:v>
       </x:c>
       <x:c r="K25" s="15" t="str">
         <x:v>https://www.serialwombat.com/p46</x:v>
@@ -1010,21 +1067,21 @@
         <x:v>25.99</x:v>
       </x:c>
       <x:c r="F26" s="3" t="str">
-        <x:v>Allowance</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="G26" s="9" t="n">
         <x:f>C26*E26</x:f>
         <x:v>25.99</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>Amazon / Nilight</x:v>
-      </x:c>
-      <x:c r="I26" s="3"/>
-      <x:c r="J26" s="3" t="str">
-        <x:v>Historical/reference price only; Amazon checkout unavailable. Confirm common negative and both color leads.</x:v>
+        <x:v>Nilight direct</x:v>
+      </x:c>
+      <x:c r="I26" s="3" t="str"/>
+      <x:c r="J26" s="24" t="str">
+        <x:v>Refs: L1, L2, L3, L4, L5, L6, L7, L8, L9, L10. Exact TL-248BW ten-pack: $25.99 observed; advertised free continental-US shipping over $19.99. Amazon price unverified. Common negative, separate blue/white positives; measure current.</x:v>
       </x:c>
       <x:c r="K26" s="15" t="str">
-        <x:v>https://www.amazon.com/Nilight-Clearance-Indicator-Trailer-Warranty/dp/B0F7XP3QZB</x:v>
+        <x:v>https://www.nilight.com/products/3-4inch-dual-color-marker-light-10pcs-blue-to-white-auxiliary-side-marker-bullet-clearance-indicator-lights-3-plug-connector-ip68-waterproof-for-trailer-truck-pickup-camper-rv-atv-utv-van-bus</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
@@ -1053,9 +1110,9 @@
       <x:c r="H27" s="22" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
-      <x:c r="I27" s="3"/>
-      <x:c r="J27" s="3" t="str">
-        <x:v>3/8-inch NPS, pulse, four wires. Possible tariff is additional; fittings and weather protection unresolved.</x:v>
+      <x:c r="I27" s="3" t="str"/>
+      <x:c r="J27" s="24" t="str">
+        <x:v>Refs: FM1. 3/8-inch NPS, pulse, four wires. Possible tariff is additional; fittings and weather protection unresolved.</x:v>
       </x:c>
       <x:c r="K27" s="15" t="str">
         <x:v>https://www.digikey.com/en/products/detail/sciosense/UFM-02-03NP4-3-8-NPS-PULSE-4-WIRE/29771278</x:v>
@@ -1075,24 +1132,24 @@
         <x:v>relay</x:v>
       </x:c>
       <x:c r="E28" s="12" t="n">
-        <x:v>2.36</x:v>
+        <x:v>1.94</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>C28*E28</x:f>
-        <x:v>2.36</x:v>
+        <x:v>1.94</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>DigiKey / Mouser</x:v>
-      </x:c>
-      <x:c r="I28" s="3"/>
-      <x:c r="J28" s="3" t="str">
-        <x:v>DigiKey backorder; check Mouser. No TQ2-L latching substitution. Footprint/pins matter.</x:v>
+        <x:v>Mouser</x:v>
+      </x:c>
+      <x:c r="I28" s="3" t="str"/>
+      <x:c r="J28" s="24" t="str">
+        <x:v>Refs: K1. Mouser showed stock at $1.94 on 7 Oct. DigiKey $2.36 backorder is an alternate. Exact nonlatching TQ2-5V only; verify physical pin orientation.</x:v>
       </x:c>
       <x:c r="K28" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/panasonic-industry/TQ2-5V/251773</x:v>
+        <x:v>https://www.mouser.com/en/ProductDetail/Panasonic-Industry/TQ2-5V?qs=HLLy2pIPwutHaTSpVfb1kw%3D%3D</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
@@ -1109,21 +1166,21 @@
         <x:v>regulator</x:v>
       </x:c>
       <x:c r="E29" s="12" t="n">
-        <x:v>0.96</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G29" s="23" t="n">
         <x:f>C29*E29</x:f>
-        <x:v>0.96</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H29" s="22" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
-      <x:c r="I29" s="3"/>
-      <x:c r="J29" s="3" t="str">
-        <x:v>Dedicated relay-coil supply only; retain specified capacitors.</x:v>
+      <x:c r="I29" s="3" t="str"/>
+      <x:c r="J29" s="24" t="str">
+        <x:v>Refs: U4. Dedicated relay-coil supply only; retain specified capacitors.</x:v>
       </x:c>
       <x:c r="K29" s="15" t="str">
         <x:v>https://www.digikey.com/en/products/detail/stmicroelectronics/L7805ABV/634711</x:v>
@@ -1142,25 +1199,26 @@
       <x:c r="D30" s="22" t="str">
         <x:v>small lot</x:v>
       </x:c>
-      <x:c r="E30" s="12" t="n">
-        <x:v>10</x:v>
+      <x:c r="E30" s="36" t="n">
+        <x:f>G75</x:f>
+        <x:v>12.459999999999999</x:v>
       </x:c>
       <x:c r="F30" s="22" t="str">
-        <x:v>Allowance</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="G30" s="23" t="n">
         <x:f>C30*E30</x:f>
-        <x:v>10</x:v>
+        <x:v>12.459999999999999</x:v>
       </x:c>
       <x:c r="H30" s="22" t="str">
-        <x:v>DigiKey / Mouser</x:v>
-      </x:c>
-      <x:c r="I30" s="3"/>
-      <x:c r="J30" s="3" t="str">
-        <x:v>Full quantities and ratings are in shopping guide and Rev D BOM. Buy small spare quantities.</x:v>
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I30" s="3" t="str"/>
+      <x:c r="J30" s="24" t="str">
+        <x:v>Linked from the detailed lots below; edit C68:C74 or E68:E74 to change spare quantities/prices. Seven exact part numbers.</x:v>
       </x:c>
       <x:c r="K30" s="15" t="str">
-        <x:v>https://www.digikey.com/</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-50FTE52-1K/9147015</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
@@ -1189,8 +1247,8 @@
       <x:c r="H31" s="3" t="str">
         <x:v>Amazon</x:v>
       </x:c>
-      <x:c r="I31" s="3"/>
-      <x:c r="J31" s="3" t="str">
+      <x:c r="I31" s="3" t="str"/>
+      <x:c r="J31" s="24" t="str">
         <x:v>Soldered carrier with secure mounting; ordinary loose Dupont jumpers are for bench use only.</x:v>
       </x:c>
       <x:c r="K31" s="15" t="str">
@@ -1223,9 +1281,9 @@
       <x:c r="H32" s="22" t="str">
         <x:v>Amazon</x:v>
       </x:c>
-      <x:c r="I32" s="3"/>
-      <x:c r="J32" s="3" t="str">
-        <x:v>Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
+      <x:c r="I32" s="3" t="str"/>
+      <x:c r="J32" s="24" t="str">
+        <x:v>Refs: TB12, TB5, TB0. Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
       </x:c>
       <x:c r="K32" s="15" t="str">
         <x:v>https://www.amazon.com/s?k=covered+barrier+terminal+block+bus+bar</x:v>
@@ -1257,8 +1315,8 @@
       <x:c r="H33" s="3" t="str">
         <x:v>Amazon</x:v>
       </x:c>
-      <x:c r="I33" s="3"/>
-      <x:c r="J33" s="3" t="str">
+      <x:c r="I33" s="3" t="str"/>
+      <x:c r="J33" s="24" t="str">
         <x:v>22 AWG signal wire planning only; load/feed gauges subject to H2. Avoid copper-clad aluminum.</x:v>
       </x:c>
       <x:c r="K33" s="15" t="str">
@@ -1291,8 +1349,8 @@
       <x:c r="H34" s="22" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
-      <x:c r="I34" s="3"/>
-      <x:c r="J34" s="3" t="str">
+      <x:c r="I34" s="3" t="str"/>
+      <x:c r="J34" s="24" t="str">
         <x:v>Measure runs first. Lamp loom needs twenty color conductors plus suitably sized common return(s).</x:v>
       </x:c>
       <x:c r="K34" s="15" t="str">
@@ -1325,8 +1383,8 @@
       <x:c r="H35" s="3" t="str">
         <x:v>Amazon / distributor</x:v>
       </x:c>
-      <x:c r="I35" s="3"/>
-      <x:c r="J35" s="3" t="str">
+      <x:c r="I35" s="3" t="str"/>
+      <x:c r="J35" s="24" t="str">
         <x:v>Use genuine rated parts with matching wire seals. Reused 14-pin machine connector excluded.</x:v>
       </x:c>
       <x:c r="K35" s="15" t="str">
@@ -1359,8 +1417,8 @@
       <x:c r="H36" s="22" t="str">
         <x:v>Amazon</x:v>
       </x:c>
-      <x:c r="I36" s="3"/>
-      <x:c r="J36" s="3" t="str">
+      <x:c r="I36" s="3" t="str"/>
+      <x:c r="J36" s="24" t="str">
         <x:v>Adhesive-lined shrink at splices; secure cable strain relief. Reduce if already owned.</x:v>
       </x:c>
       <x:c r="K36" s="15" t="str">
@@ -1393,8 +1451,8 @@
       <x:c r="H37" s="3" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
-      <x:c r="I37" s="3"/>
-      <x:c r="J37" s="3" t="str">
+      <x:c r="I37" s="3" t="str"/>
+      <x:c r="J37" s="24" t="str">
         <x:v>Insulated board clearance above steel plate; mounting should not puncture the sealing cavity.</x:v>
       </x:c>
       <x:c r="K37" s="15" t="str">
@@ -1427,8 +1485,8 @@
       <x:c r="H38" s="22" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
-      <x:c r="I38" s="3"/>
-      <x:c r="J38" s="3" t="str">
+      <x:c r="I38" s="3" t="str"/>
+      <x:c r="J38" s="24" t="str">
         <x:v>Nominal 240 x 160 x 90 mm. Preferred planning size; confirm physical layout before drilling.</x:v>
       </x:c>
       <x:c r="K38" s="15" t="str">
@@ -1461,8 +1519,8 @@
       <x:c r="H39" s="3" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
-      <x:c r="I39" s="3"/>
-      <x:c r="J39" s="3" t="str">
+      <x:c r="I39" s="3" t="str"/>
+      <x:c r="J39" s="24" t="str">
         <x:v>Box plus plate clears advertised $49 free-shipping threshold; checkout confirmation still required.</x:v>
       </x:c>
       <x:c r="K39" s="15" t="str">
@@ -1495,8 +1553,8 @@
       <x:c r="H40" s="22" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
-      <x:c r="I40" s="3"/>
-      <x:c r="J40" s="3" t="str">
+      <x:c r="I40" s="3" t="str"/>
+      <x:c r="J40" s="24" t="str">
         <x:v>M12 x 1.5; jacket OD 3–6.5 mm. Use only where cable diameter fits; mounting hardware included.</x:v>
       </x:c>
       <x:c r="K40" s="15" t="str">
@@ -1529,8 +1587,8 @@
       <x:c r="H41" s="3" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
-      <x:c r="I41" s="3"/>
-      <x:c r="J41" s="3" t="str">
+      <x:c r="I41" s="3" t="str"/>
+      <x:c r="J41" s="24" t="str">
         <x:v>Machine/display cable may need larger glands or matched multi-hole inserts; measure first.</x:v>
       </x:c>
       <x:c r="K41" s="15" t="str">
@@ -1563,8 +1621,8 @@
       <x:c r="H42" s="22" t="str">
         <x:v>Local / Amazon</x:v>
       </x:c>
-      <x:c r="I42" s="3"/>
-      <x:c r="J42" s="3" t="str">
+      <x:c r="I42" s="3" t="str"/>
+      <x:c r="J42" s="24" t="str">
         <x:v>Plan approximately 300 mm long; verify actual grommet diameter/pitch. No rated finished housing selected.</x:v>
       </x:c>
       <x:c r="K42" s="15" t="str">
@@ -1597,8 +1655,8 @@
       <x:c r="H43" s="3" t="str">
         <x:v>Local / distributor</x:v>
       </x:c>
-      <x:c r="I43" s="3"/>
-      <x:c r="J43" s="3" t="str">
+      <x:c r="I43" s="3" t="str"/>
+      <x:c r="J43" s="24" t="str">
         <x:v>Dedicated splash/impact protection, supported plumbing and sealed terminations; exact housing pending geometry.</x:v>
       </x:c>
       <x:c r="K43" s="15" t="str">
@@ -1631,8 +1689,8 @@
       <x:c r="H44" s="22" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
-      <x:c r="I44" s="3"/>
-      <x:c r="J44" s="3" t="str">
+      <x:c r="I44" s="3" t="str"/>
+      <x:c r="J44" s="24" t="str">
         <x:v>Reuse existing suitable items; select pressure rating and mesh for nozzle/meter requirements.</x:v>
       </x:c>
       <x:c r="K44" s="15" t="str">
@@ -1665,8 +1723,8 @@
       <x:c r="H45" s="3" t="str">
         <x:v>Plumbing supplier</x:v>
       </x:c>
-      <x:c r="I45" s="3"/>
-      <x:c r="J45" s="3" t="str">
+      <x:c r="I45" s="3" t="str"/>
+      <x:c r="J45" s="24" t="str">
         <x:v>PROCUREMENT HOLD: straight NPS thread and actual seal geometry must match; NPT or cone-seat swivel is not assumed compatible.</x:v>
       </x:c>
       <x:c r="K45" s="15" t="str">
@@ -1699,8 +1757,8 @@
       <x:c r="H46" s="22" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
-      <x:c r="I46" s="3"/>
-      <x:c r="J46" s="3" t="str">
+      <x:c r="I46" s="3" t="str"/>
+      <x:c r="J46" s="24" t="str">
         <x:v>US garden hose thread is 3/4 GHT, distinct from 1/2 NPT valve threads. Include removable unions as required.</x:v>
       </x:c>
       <x:c r="K46" s="15" t="str">
@@ -1733,8 +1791,8 @@
       <x:c r="H47" s="3" t="str">
         <x:v>Local</x:v>
       </x:c>
-      <x:c r="I47" s="3"/>
-      <x:c r="J47" s="3" t="str">
+      <x:c r="I47" s="3" t="str"/>
+      <x:c r="J47" s="24" t="str">
         <x:v>Respect meter straight lengths and seal type. Do not seal NPS solely with PTFE tape.</x:v>
       </x:c>
       <x:c r="K47" s="15" t="str">
@@ -1767,8 +1825,8 @@
       <x:c r="H48" s="22" t="str">
         <x:v>Amazon / distributor</x:v>
       </x:c>
-      <x:c r="I48" s="3"/>
-      <x:c r="J48" s="3" t="str">
+      <x:c r="I48" s="3" t="str"/>
+      <x:c r="J48" s="24" t="str">
         <x:v>Later, after testing; mask contacts, connectors and vents. Not a substitute for the gasketed box.</x:v>
       </x:c>
       <x:c r="K48" s="15" t="str">
@@ -1801,8 +1859,8 @@
       <x:c r="H49" s="3" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
-      <x:c r="I49" s="3"/>
-      <x:c r="J49" s="3" t="str">
+      <x:c r="I49" s="3" t="str"/>
+      <x:c r="J49" s="24" t="str">
         <x:v>Bench only, close to battery; size fuse to test stage and weakest wire. Not a new machine fuse block.</x:v>
       </x:c>
       <x:c r="K49" s="15" t="str">
@@ -1823,24 +1881,24 @@
         <x:v>resistor allowance</x:v>
       </x:c>
       <x:c r="E50" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3.36</x:v>
       </x:c>
       <x:c r="F50" s="22" t="str">
-        <x:v>Allowance</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="G50" s="23" t="n">
         <x:f>C50*E50</x:f>
-        <x:v>2</x:v>
+        <x:v>3.36</x:v>
       </x:c>
       <x:c r="H50" s="22" t="str">
-        <x:v>DigiKey / Mouser</x:v>
-      </x:c>
-      <x:c r="I50" s="3"/>
-      <x:c r="J50" s="3" t="str">
-        <x:v>DAC test load only. Expected 1/3/5 V at 4/12/20 mA; remove before valve wiring.</x:v>
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I50" s="3" t="str"/>
+      <x:c r="J50" s="24" t="str">
+        <x:v>Vishay RN65E2500BB14: 250 ohm, 0.1%, 0.5 W. Removable DAC bench load only; never add as a permanent valve/feedback shunt.</x:v>
       </x:c>
       <x:c r="K50" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products?keywords=250%20ohm%200.1%25%200.5W%20resistor</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/vishay-dale/RN65E2500BB14/3193953</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
@@ -1869,8 +1927,8 @@
       <x:c r="H51" s="3" t="str">
         <x:v>Amazon / existing</x:v>
       </x:c>
-      <x:c r="I51" s="3"/>
-      <x:c r="J51" s="3" t="str">
+      <x:c r="I51" s="3" t="str"/>
+      <x:c r="J51" s="24" t="str">
         <x:v>Set quantity to zero if owned. Must carry data, not charging-only.</x:v>
       </x:c>
       <x:c r="K51" s="15" t="str">
@@ -1903,9 +1961,9 @@
       <x:c r="J53" s="3"/>
       <x:c r="K53" s="3"/>
     </x:row>
-    <x:row r="54" ht="26" customHeight="1">
-      <x:c r="A54" s="3" t="str">
-        <x:v>Shipping is added once per supplier basket below. All rates are assumptions except the conditional free-shipping offer.</x:v>
+    <x:row r="54" ht="32" customHeight="1">
+      <x:c r="A54" s="24" t="str">
+        <x:v>Shipping is budgeted once per supplier basket. AutomationDirect and Nilight have conditional free-shipping offers.</x:v>
       </x:c>
       <x:c r="B54" s="3"/>
       <x:c r="C54" s="3"/>
@@ -1962,7 +2020,7 @@
       <x:c r="G57" s="3"/>
       <x:c r="H57" s="3"/>
       <x:c r="I57" s="3"/>
-      <x:c r="J57" s="3" t="str">
+      <x:c r="J57" s="24" t="str">
         <x:v>Allowance; weight-based checkout quote unavailable</x:v>
       </x:c>
       <x:c r="K57" s="15" t="str">
@@ -1983,7 +2041,7 @@
       <x:c r="G58" s="3"/>
       <x:c r="H58" s="3"/>
       <x:c r="I58" s="3"/>
-      <x:c r="J58" s="3" t="str">
+      <x:c r="J58" s="24" t="str">
         <x:v>Allowance; combine Nano and both opto boards</x:v>
       </x:c>
       <x:c r="K58" s="15" t="str">
@@ -2004,7 +2062,7 @@
       <x:c r="G59" s="3"/>
       <x:c r="H59" s="3"/>
       <x:c r="I59" s="3"/>
-      <x:c r="J59" s="3" t="str">
+      <x:c r="J59" s="24" t="str">
         <x:v>Allowance; combine both modules; shipping resumes Oct 8</x:v>
       </x:c>
       <x:c r="K59" s="15" t="str">
@@ -2014,22 +2072,22 @@
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" s="3"/>
       <x:c r="B60" s="3" t="str">
-        <x:v>DigiKey / possible Mouser split</x:v>
+        <x:v>DigiKey + Mouser</x:v>
       </x:c>
       <x:c r="C60" s="3"/>
       <x:c r="D60" s="3"/>
       <x:c r="E60" s="12" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F60" s="3"/>
       <x:c r="G60" s="3"/>
       <x:c r="H60" s="3"/>
       <x:c r="I60" s="3"/>
-      <x:c r="J60" s="3" t="str">
-        <x:v>Allowance; DigiKey advertises rates from $4.99, not a basket quote</x:v>
+      <x:c r="J60" s="24" t="str">
+        <x:v>Combined allowance for two supplier baskets; neither is a destination quote</x:v>
       </x:c>
       <x:c r="K60" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/panasonic-industry/TQ2-5V/251773</x:v>
+        <x:v>https://www.mouser.com/en/ProductDetail/Panasonic-Industry/TQ2-5V?qs=HLLy2pIPwutHaTSpVfb1kw%3D%3D</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
@@ -2046,7 +2104,7 @@
       <x:c r="G61" s="3"/>
       <x:c r="H61" s="3"/>
       <x:c r="I61" s="3"/>
-      <x:c r="J61" s="3" t="str">
+      <x:c r="J61" s="24" t="str">
         <x:v>Advertised free shipping over $49; assumed eligible box/plate/glands basket</x:v>
       </x:c>
       <x:c r="K61" s="15" t="str">
@@ -2067,8 +2125,8 @@
       <x:c r="G62" s="3"/>
       <x:c r="H62" s="3"/>
       <x:c r="I62" s="3"/>
-      <x:c r="J62" s="3" t="str">
-        <x:v>Allowance; Prime and seller shipping are not verified</x:v>
+      <x:c r="J62" s="24" t="str">
+        <x:v>Allowance for Amazon/local/other purchases. Nilight advertises free continental-US shipping over $19.99; no additional lamp shipping included.</x:v>
       </x:c>
       <x:c r="K62" s="15" t="str">
         <x:v>https://www.amazon.com/</x:v>
@@ -2101,7 +2159,9 @@
       <x:c r="K64" s="3"/>
     </x:row>
     <x:row r="65" ht="26" customHeight="1">
-      <x:c r="A65" s="3"/>
+      <x:c r="A65" s="24" t="str">
+        <x:v>Exact small parts · linked to the main basket; purchase quantities include spares.</x:v>
+      </x:c>
       <x:c r="B65" s="3"/>
       <x:c r="C65" s="3"/>
       <x:c r="D65" s="3"/>
@@ -2114,30 +2174,310 @@
       <x:c r="K65" s="3"/>
     </x:row>
     <x:row r="66" ht="26" customHeight="1">
-      <x:c r="A66" s="3"/>
-      <x:c r="B66" s="3"/>
-      <x:c r="C66" s="3"/>
-      <x:c r="D66" s="3"/>
-      <x:c r="E66" s="3"/>
-      <x:c r="F66" s="3"/>
-      <x:c r="G66" s="3"/>
-      <x:c r="H66" s="3"/>
+      <x:c r="A66" s="20" t="str">
+        <x:v>Installed quantities match Rev D. Reused X1 costs $0. The separate 250-ohm test resistor is on row 50.</x:v>
+      </x:c>
+      <x:c r="B66" s="20"/>
+      <x:c r="C66" s="20"/>
+      <x:c r="D66" s="20"/>
+      <x:c r="E66" s="20"/>
+      <x:c r="F66" s="20"/>
+      <x:c r="G66" s="20"/>
+      <x:c r="H66" s="20"/>
       <x:c r="I66" s="3"/>
       <x:c r="J66" s="3"/>
       <x:c r="K66" s="3"/>
     </x:row>
     <x:row r="67" ht="26" customHeight="1">
-      <x:c r="A67" s="3"/>
-      <x:c r="B67" s="3"/>
-      <x:c r="C67" s="3"/>
-      <x:c r="D67" s="3"/>
-      <x:c r="E67" s="3"/>
-      <x:c r="F67" s="3"/>
-      <x:c r="G67" s="3"/>
-      <x:c r="H67" s="3"/>
-      <x:c r="I67" s="3"/>
-      <x:c r="J67" s="3"/>
-      <x:c r="K67" s="3"/>
+      <x:c r="A67" s="18" t="str">
+        <x:v>References</x:v>
+      </x:c>
+      <x:c r="B67" s="18" t="str">
+        <x:v>Exact part number</x:v>
+      </x:c>
+      <x:c r="C67" s="18" t="str">
+        <x:v>Buy qty</x:v>
+      </x:c>
+      <x:c r="D67" s="18" t="str">
+        <x:v>Installed</x:v>
+      </x:c>
+      <x:c r="E67" s="18" t="str">
+        <x:v>Unit USD</x:v>
+      </x:c>
+      <x:c r="F67" s="18" t="str">
+        <x:v>Price basis</x:v>
+      </x:c>
+      <x:c r="G67" s="18" t="str">
+        <x:v>Lot USD</x:v>
+      </x:c>
+      <x:c r="H67" s="18" t="str">
+        <x:v>Vendor</x:v>
+      </x:c>
+      <x:c r="I67" s="3" t="str"/>
+      <x:c r="J67" s="3" t="str">
+        <x:v>Specification / notes</x:v>
+      </x:c>
+      <x:c r="K67" s="3" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="66" customHeight="1">
+      <x:c r="A68" s="24" t="str">
+        <x:v>R1, R2, R3, R4, R8, R9</x:v>
+      </x:c>
+      <x:c r="B68" s="24" t="str">
+        <x:v>MFR-50FTE52-1K</x:v>
+      </x:c>
+      <x:c r="C68" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D68" s="31" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E68" s="30" t="n">
+        <x:v>0.076</x:v>
+      </x:c>
+      <x:c r="F68" s="24" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G68" s="27" t="n">
+        <x:f>C68*E68</x:f>
+        <x:v>0.76</x:v>
+      </x:c>
+      <x:c r="H68" s="24" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I68" s="24" t="str"/>
+      <x:c r="J68" s="24" t="str">
+        <x:v>1 kohm, 1%, 0.5 W axial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K68" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-50FTE52-1K/9147015</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="66" customHeight="1">
+      <x:c r="A69" s="28" t="str">
+        <x:v>R5</x:v>
+      </x:c>
+      <x:c r="B69" s="28" t="str">
+        <x:v>MFR-25FBF52-100K</x:v>
+      </x:c>
+      <x:c r="C69" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D69" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E69" s="30" t="n">
+        <x:v>0.042</x:v>
+      </x:c>
+      <x:c r="F69" s="28" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G69" s="29" t="n">
+        <x:f>C69*E69</x:f>
+        <x:v>0.42000000000000004</x:v>
+      </x:c>
+      <x:c r="H69" s="28" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I69" s="24" t="str"/>
+      <x:c r="J69" s="24" t="str">
+        <x:v>100 kohm, 1%, 0.25 W axial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K69" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-100K/13473</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="66" customHeight="1">
+      <x:c r="A70" s="24" t="str">
+        <x:v>R6, R7</x:v>
+      </x:c>
+      <x:c r="B70" s="24" t="str">
+        <x:v>MFR-25FBF52-4K7</x:v>
+      </x:c>
+      <x:c r="C70" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D70" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E70" s="30" t="n">
+        <x:v>0.044</x:v>
+      </x:c>
+      <x:c r="F70" s="24" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G70" s="27" t="n">
+        <x:f>C70*E70</x:f>
+        <x:v>0.43999999999999995</x:v>
+      </x:c>
+      <x:c r="H70" s="24" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I70" s="24" t="str"/>
+      <x:c r="J70" s="24" t="str">
+        <x:v>4.7 kohm, 1%, 0.25 W axial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K70" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-4K7/9138176</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="66" customHeight="1">
+      <x:c r="A71" s="28" t="str">
+        <x:v>D1, D2, D3, D4</x:v>
+      </x:c>
+      <x:c r="B71" s="28" t="str">
+        <x:v>1N4148 (onsemi)</x:v>
+      </x:c>
+      <x:c r="C71" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D71" s="32" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E71" s="30" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="F71" s="28" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G71" s="29" t="n">
+        <x:f>C71*E71</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="H71" s="28" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I71" s="24" t="str"/>
+      <x:c r="J71" s="24" t="str">
+        <x:v>1N4148 axial DO-35; band = cathode; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K71" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/onsemi/1N4148/458603</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="66" customHeight="1">
+      <x:c r="A72" s="24" t="str">
+        <x:v>C1, C2, C5, C10, C11, C12</x:v>
+      </x:c>
+      <x:c r="B72" s="24" t="str">
+        <x:v>C315C104K5R5TA</x:v>
+      </x:c>
+      <x:c r="C72" s="25" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D72" s="31" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E72" s="30" t="n">
+        <x:v>0.488</x:v>
+      </x:c>
+      <x:c r="F72" s="24" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G72" s="27" t="n">
+        <x:f>C72*E72</x:f>
+        <x:v>4.88</x:v>
+      </x:c>
+      <x:c r="H72" s="24" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I72" s="24" t="str"/>
+      <x:c r="J72" s="24" t="str">
+        <x:v>100 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K72" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/kemet/C315C104K5R5TA/12701330</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="66" customHeight="1">
+      <x:c r="A73" s="28" t="str">
+        <x:v>C4</x:v>
+      </x:c>
+      <x:c r="B73" s="28" t="str">
+        <x:v>SR305C334KARTR1</x:v>
+      </x:c>
+      <x:c r="C73" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D73" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E73" s="30" t="n">
+        <x:v>1.48</x:v>
+      </x:c>
+      <x:c r="F73" s="28" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G73" s="29" t="n">
+        <x:f>C73*E73</x:f>
+        <x:v>2.96</x:v>
+      </x:c>
+      <x:c r="H73" s="28" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I73" s="24" t="str"/>
+      <x:c r="J73" s="24" t="str">
+        <x:v>330 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K73" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/kyocera-avx/SR305C334KARTR1/9948632</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="66" customHeight="1">
+      <x:c r="A74" s="24" t="str">
+        <x:v>C7, C8, C9</x:v>
+      </x:c>
+      <x:c r="B74" s="24" t="str">
+        <x:v>EEU-FC1V470B</x:v>
+      </x:c>
+      <x:c r="C74" s="25" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D74" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E74" s="30" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="F74" s="24" t="str">
+        <x:v>Published</x:v>
+      </x:c>
+      <x:c r="G74" s="27" t="n">
+        <x:f>C74*E74</x:f>
+        <x:v>2.4</x:v>
+      </x:c>
+      <x:c r="H74" s="24" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="I74" s="24" t="str"/>
+      <x:c r="J74" s="24" t="str">
+        <x:v>47 uF, 35 V, 105 C, polarized radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+      </x:c>
+      <x:c r="K74" s="15" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/panasonic-industry/EEU-FC1V470B/16639056</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="18" t="str"/>
+      <x:c r="B75" s="18" t="str"/>
+      <x:c r="C75" s="18" t="str"/>
+      <x:c r="D75" s="18" t="str"/>
+      <x:c r="E75" s="18" t="str"/>
+      <x:c r="F75" s="18" t="str">
+        <x:v>Lot total</x:v>
+      </x:c>
+      <x:c r="G75" s="33" t="n">
+        <x:f>SUM(G68:G74)</x:f>
+        <x:v>12.459999999999999</x:v>
+      </x:c>
+      <x:c r="H75" s="18" t="str"/>
+      <x:c r="I75" s="3" t="str"/>
+      <x:c r="J75" s="3" t="str">
+        <x:v>Included once through E30. No extra fee or shipping added here.</x:v>
+      </x:c>
+      <x:c r="K75" s="3" t="str"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F20:F52">
@@ -2287,8 +2627,8 @@
       <x:c r="G7" s="3"/>
       <x:c r="H7" s="3"/>
       <x:c r="I7" s="3"/>
-      <x:c r="J7" s="3" t="str">
-        <x:v>200 x 120 x 90 mm; consider only after measured two-level layout. Plate extra; smaller is harder to wire/service.</x:v>
+      <x:c r="J7" s="24" t="str">
+        <x:v>200 x 120 x 91 mm; consider only after measured two-level layout. Plate extra; smaller is harder to wire/service.</x:v>
       </x:c>
       <x:c r="K7" s="15" t="str">
         <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/miniature_cases/1554u2gy</x:v>
@@ -2312,7 +2652,7 @@
       <x:c r="G8" s="22"/>
       <x:c r="H8" s="22"/>
       <x:c r="I8" s="3"/>
-      <x:c r="J8" s="3" t="str">
+      <x:c r="J8" s="24" t="str">
         <x:v>Same exact ABX00028; $0.80 cheaper but separate shipping may cost more.</x:v>
       </x:c>
       <x:c r="K8" s="15" t="str">
@@ -2337,7 +2677,7 @@
       <x:c r="G9" s="3"/>
       <x:c r="H9" s="3"/>
       <x:c r="I9" s="3"/>
-      <x:c r="J9" s="3" t="str">
+      <x:c r="J9" s="24" t="str">
         <x:v>CC/CV. Advertised DPS154 code subtracts $4 if accepted. Requires suitable higher-voltage DC/USB-C PD input; not an all-in-one AC supply.</x:v>
       </x:c>
       <x:c r="K9" s="15" t="str">
@@ -2362,7 +2702,7 @@
       <x:c r="G10" s="22"/>
       <x:c r="H10" s="22"/>
       <x:c r="I10" s="3"/>
-      <x:c r="J10" s="3" t="str">
+      <x:c r="J10" s="24" t="str">
         <x:v>Simpler all-in-one option if 110/120 V US version is near $60. Adjustable CC/CV; 10 A rating is not the current-limit setting.</x:v>
       </x:c>
       <x:c r="K10" s="15" t="str">
@@ -2382,12 +2722,12 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>Published; manufacturer out of stock</x:v>
+        <x:v>Published 4 Oct; out of stock at that review; excluded comparison only</x:v>
       </x:c>
       <x:c r="G11" s="3"/>
       <x:c r="H11" s="3"/>
       <x:c r="I11" s="3"/>
-      <x:c r="J11" s="3" t="str">
+      <x:c r="J11" s="24" t="str">
         <x:v>Eight high-side channels, but not a drop-in: different interface, extra I/O hardware and watchdog/diagnostic redesign. Do not buy as a substitute.</x:v>
       </x:c>
       <x:c r="K11" s="15" t="str">
@@ -2407,12 +2747,12 @@
         <x:v>9.9</x:v>
       </x:c>
       <x:c r="F12" s="22" t="str">
-        <x:v>Published comparison price</x:v>
+        <x:v>Published comparison price observed 4 Oct; excluded option</x:v>
       </x:c>
       <x:c r="G12" s="22"/>
       <x:c r="H12" s="22"/>
       <x:c r="I12" s="3"/>
-      <x:c r="J12" s="3" t="str">
+      <x:c r="J12" s="24" t="str">
         <x:v>Not selected: 18–24 V power requirement adds another converter to this nominal-12 V project.</x:v>
       </x:c>
       <x:c r="K12" s="15" t="str">
@@ -2437,7 +2777,7 @@
       <x:c r="G13" s="3"/>
       <x:c r="H13" s="3"/>
       <x:c r="I13" s="3"/>
-      <x:c r="J13" s="3" t="str">
+      <x:c r="J13" s="24" t="str">
         <x:v>Includes suitable tip/stand; buy electronics solder and flux, not plumbing acid flux.</x:v>
       </x:c>
       <x:c r="K13" s="15" t="str">
@@ -2462,7 +2802,7 @@
       <x:c r="G14" s="22"/>
       <x:c r="H14" s="22"/>
       <x:c r="I14" s="3"/>
-      <x:c r="J14" s="3" t="str">
+      <x:c r="J14" s="24" t="str">
         <x:v>Match crimper to chosen contacts/ferrules. Ordinary pliers do not replace the correct contact crimp tool.</x:v>
       </x:c>
       <x:c r="K14" s="15" t="str">
@@ -2487,7 +2827,7 @@
       <x:c r="G15" s="3"/>
       <x:c r="H15" s="3"/>
       <x:c r="I15" s="3"/>
-      <x:c r="J15" s="3" t="str">
+      <x:c r="J15" s="24" t="str">
         <x:v>Allow complete cleaning/drying before coating. Reuse existing suitable supplies.</x:v>
       </x:c>
       <x:c r="K15" s="15" t="str">

</xml_diff>

<commit_message>
Remove permanent flow meter in Revision E and document power-off input behavior
</commit_message>
<xml_diff>
--- a/docs/assets/procurement/shopping-list.xlsx
+++ b/docs/assets/procurement/shopping-list.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="R01d9dcc738004bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="Rcedf89cffe184b1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shopping" sheetId="1" r:id="R1b3fdb678cfe403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="2" r:id="R329aa51af37a4858"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -76,7 +76,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -106,6 +106,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8F0F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -139,7 +149,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -245,6 +255,15 @@
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -520,7 +539,7 @@
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Revision D · prices reviewed 7 October 2026 · USD planning budget; no temperature probes.</x:v>
+        <x:v>Revision E · no flow / temperature sensors · retained prices reviewed 7 October 2026.</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
@@ -552,7 +571,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>SUM(G20:G52)</x:f>
-        <x:v>613</x:v>
+        <x:v>517.9</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="18" t="str">
@@ -606,7 +625,7 @@
       </x:c>
       <x:c r="E8" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D8)</x:f>
-        <x:v>227.95</x:v>
+        <x:v>148.29000000000002</x:v>
       </x:c>
       <x:c r="F8" s="3"/>
       <x:c r="G8" s="3"/>
@@ -654,7 +673,7 @@
       </x:c>
       <x:c r="E10" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D10)</x:f>
-        <x:v>87.46000000000001</x:v>
+        <x:v>87.02000000000001</x:v>
       </x:c>
       <x:c r="F10" s="3"/>
       <x:c r="G10" s="3"/>
@@ -673,7 +692,7 @@
       </x:c>
       <x:c r="B11" s="9" t="n">
         <x:f>ROUND((SUM(B6:B8)-B9)*B10,2)</x:f>
-        <x:v>56.84</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3" t="str">
@@ -681,7 +700,7 @@
       </x:c>
       <x:c r="E11" s="9" t="n">
         <x:f>SUMIFS($G$20:$G$52,$A$20:$A$52,D11)</x:f>
-        <x:v>114</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="F11" s="3"/>
       <x:c r="G11" s="3"/>
@@ -700,7 +719,7 @@
       </x:c>
       <x:c r="B12" s="10" t="n">
         <x:f>SUM(B6:B8)-B9+B11</x:f>
-        <x:v>745.84</x:v>
+        <x:v>642.9</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3" t="str">
@@ -715,7 +734,7 @@
       <x:c r="H12" s="3"/>
       <x:c r="I12" s="3"/>
       <x:c r="J12" s="3" t="str">
-        <x:v>Driver availability, meter adapters, physical fit and hardware qualification remain unresolved.</x:v>
+        <x:v>Driver availability, valve interface qualification, physical fit and hardware testing remain unresolved. No meter adapters are required.</x:v>
       </x:c>
       <x:c r="K12" s="3"/>
     </x:row>
@@ -738,7 +757,7 @@
       </x:c>
       <x:c r="B14" s="9" t="n">
         <x:f>SUMIFS(G20:G52,F20:F52,"Published")</x:f>
-        <x:v>312.00000000000006</x:v>
+        <x:v>251.90000000000006</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
@@ -758,7 +777,7 @@
       </x:c>
       <x:c r="B15" s="9" t="n">
         <x:f>SUMIFS(G20:G52,F20:F52,"Allowance")</x:f>
-        <x:v>301</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="C15" s="3"/>
       <x:c r="D15" s="3"/>
@@ -1086,36 +1105,36 @@
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" s="22" t="str">
-        <x:v>Water</x:v>
+        <x:v>Control</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>ScioSense UFM-02-03NP4</x:v>
+        <x:v>Panasonic TQ2-5V nonlatching DPDT</x:v>
       </x:c>
       <x:c r="C27" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D27" s="22" t="str">
-        <x:v>meter</x:v>
+        <x:v>relay</x:v>
       </x:c>
       <x:c r="E27" s="12" t="n">
-        <x:v>59.66</x:v>
+        <x:v>1.94</x:v>
       </x:c>
       <x:c r="F27" s="22" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G27" s="23" t="n">
         <x:f>C27*E27</x:f>
-        <x:v>59.66</x:v>
+        <x:v>1.94</x:v>
       </x:c>
       <x:c r="H27" s="22" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>Mouser</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str"/>
       <x:c r="J27" s="24" t="str">
-        <x:v>Refs: FM1. 3/8-inch NPS, pulse, four wires. Possible tariff is additional; fittings and weather protection unresolved.</x:v>
+        <x:v>Refs: K1. Mouser showed stock at $1.94 on 7 Oct. DigiKey $2.36 backorder is an alternate. Exact nonlatching TQ2-5V only; verify physical pin orientation.</x:v>
       </x:c>
       <x:c r="K27" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/sciosense/UFM-02-03NP4-3-8-NPS-PULSE-4-WIRE/29771278</x:v>
+        <x:v>https://www.mouser.com/en/ProductDetail/Panasonic-Industry/TQ2-5V?qs=HLLy2pIPwutHaTSpVfb1kw%3D%3D</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
@@ -1123,67 +1142,68 @@
         <x:v>Control</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>Panasonic TQ2-5V nonlatching DPDT</x:v>
+        <x:v>ST L7805ABV TO-220</x:v>
       </x:c>
       <x:c r="C28" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>relay</x:v>
+        <x:v>regulator</x:v>
       </x:c>
       <x:c r="E28" s="12" t="n">
-        <x:v>1.94</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G28" s="9" t="n">
         <x:f>C28*E28</x:f>
-        <x:v>1.94</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Mouser</x:v>
+        <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str"/>
       <x:c r="J28" s="24" t="str">
-        <x:v>Refs: K1. Mouser showed stock at $1.94 on 7 Oct. DigiKey $2.36 backorder is an alternate. Exact nonlatching TQ2-5V only; verify physical pin orientation.</x:v>
+        <x:v>Refs: U4. Dedicated relay-coil supply only; retain specified capacitors.</x:v>
       </x:c>
       <x:c r="K28" s="15" t="str">
-        <x:v>https://www.mouser.com/en/ProductDetail/Panasonic-Industry/TQ2-5V?qs=HLLy2pIPwutHaTSpVfb1kw%3D%3D</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/stmicroelectronics/L7805ABV/634711</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" s="22" t="str">
-        <x:v>Control</x:v>
+        <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>ST L7805ABV TO-220</x:v>
+        <x:v>Exact resistors, diodes and capacitors</x:v>
       </x:c>
       <x:c r="C29" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D29" s="22" t="str">
-        <x:v>regulator</x:v>
-      </x:c>
-      <x:c r="E29" s="12" t="n">
-        <x:v>0.9</x:v>
+        <x:v>small lot</x:v>
+      </x:c>
+      <x:c r="E29" s="38" t="n">
+        <x:f>G75</x:f>
+        <x:v>12.020000000000001</x:v>
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G29" s="23" t="n">
         <x:f>C29*E29</x:f>
-        <x:v>0.9</x:v>
+        <x:v>12.020000000000001</x:v>
       </x:c>
       <x:c r="H29" s="22" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str"/>
       <x:c r="J29" s="24" t="str">
-        <x:v>Refs: U4. Dedicated relay-coil supply only; retain specified capacitors.</x:v>
+        <x:v>Linked from the detailed lots below; edit C68:C73 or E68:E73 to change spare quantities/prices. Six exact part numbers.</x:v>
       </x:c>
       <x:c r="K29" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/stmicroelectronics/L7805ABV/634711</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-50FTE52-1K/9147015</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
@@ -1191,34 +1211,33 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>Exact resistors, diodes and capacitors</x:v>
+        <x:v>FR4 perfboard, Nano headers and sockets</x:v>
       </x:c>
       <x:c r="C30" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="22" t="str">
-        <x:v>small lot</x:v>
-      </x:c>
-      <x:c r="E30" s="36" t="n">
-        <x:f>G75</x:f>
-        <x:v>12.459999999999999</x:v>
+        <x:v>set</x:v>
+      </x:c>
+      <x:c r="E30" s="39" t="n">
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F30" s="22" t="str">
-        <x:v>Published</x:v>
+        <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G30" s="23" t="n">
         <x:f>C30*E30</x:f>
-        <x:v>12.459999999999999</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H30" s="22" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str"/>
       <x:c r="J30" s="24" t="str">
-        <x:v>Linked from the detailed lots below; edit C68:C74 or E68:E74 to change spare quantities/prices. Seven exact part numbers.</x:v>
+        <x:v>Soldered carrier with secure mounting; ordinary loose Dupont jumpers are for bench use only.</x:v>
       </x:c>
       <x:c r="K30" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-50FTE52-1K/9147015</x:v>
+        <x:v>https://www.amazon.com/s?k=FR4+perfboard+2.54mm+headers+female+socket</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
@@ -1226,7 +1245,7 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>FR4 perfboard, Nano headers and sockets</x:v>
+        <x:v>12 V, 5 V and ground distribution terminals</x:v>
       </x:c>
       <x:c r="C31" s="21" t="n">
         <x:v>1</x:v>
@@ -1235,24 +1254,24 @@
         <x:v>set</x:v>
       </x:c>
       <x:c r="E31" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G31" s="9" t="n">
         <x:f>C31*E31</x:f>
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
         <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str"/>
       <x:c r="J31" s="24" t="str">
-        <x:v>Soldered carrier with secure mounting; ordinary loose Dupont jumpers are for bench use only.</x:v>
+        <x:v>Refs: TB12, TB5, TB0. Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
       </x:c>
       <x:c r="K31" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=FR4+perfboard+2.54mm+headers+female+socket</x:v>
+        <x:v>https://www.amazon.com/s?k=covered+barrier+terminal+block+bus+bar</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
@@ -1260,13 +1279,13 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B32" s="22" t="str">
-        <x:v>12 V, 5 V and ground distribution terminals</x:v>
+        <x:v>Stranded copper internal hookup wire</x:v>
       </x:c>
       <x:c r="C32" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D32" s="22" t="str">
-        <x:v>set</x:v>
+        <x:v>assortment</x:v>
       </x:c>
       <x:c r="E32" s="12" t="n">
         <x:v>10</x:v>
@@ -1283,10 +1302,10 @@
       </x:c>
       <x:c r="I32" s="3" t="str"/>
       <x:c r="J32" s="24" t="str">
-        <x:v>Refs: TB12, TB5, TB0. Three separate labeled buses. Quantity depends on harness layout; size to verified fuse and loads.</x:v>
+        <x:v>22 AWG signal wire planning only; load/feed gauges subject to H2. Avoid copper-clad aluminum.</x:v>
       </x:c>
       <x:c r="K32" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=covered+barrier+terminal+block+bus+bar</x:v>
+        <x:v>https://www.amazon.com/s?k=stranded+copper+hookup+wire+22+awg+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
@@ -1294,33 +1313,33 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
-        <x:v>Stranded copper internal hookup wire</x:v>
+        <x:v>Jacketed outdoor harness cable</x:v>
       </x:c>
       <x:c r="C33" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D33" s="3" t="str">
-        <x:v>assortment</x:v>
+        <x:v>length allowance</x:v>
       </x:c>
       <x:c r="E33" s="12" t="n">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F33" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G33" s="9" t="n">
         <x:f>C33*E33</x:f>
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H33" s="3" t="str">
-        <x:v>Amazon</x:v>
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str"/>
       <x:c r="J33" s="24" t="str">
-        <x:v>22 AWG signal wire planning only; load/feed gauges subject to H2. Avoid copper-clad aluminum.</x:v>
+        <x:v>Measure runs first. Lamp loom needs twenty color conductors plus suitably sized common return(s).</x:v>
       </x:c>
       <x:c r="K33" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=stranded+copper+hookup+wire+22+awg+kit</x:v>
+        <x:v>https://www.amazon.com/s?k=outdoor+multiconductor+copper+control+cable</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
@@ -1328,33 +1347,33 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>Jacketed outdoor harness cable</x:v>
+        <x:v>Locking sealed cable connectors</x:v>
       </x:c>
       <x:c r="C34" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D34" s="22" t="str">
-        <x:v>length allowance</x:v>
+        <x:v>set</x:v>
       </x:c>
       <x:c r="E34" s="12" t="n">
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F34" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G34" s="23" t="n">
         <x:f>C34*E34</x:f>
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H34" s="22" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>Amazon / distributor</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str"/>
       <x:c r="J34" s="24" t="str">
-        <x:v>Measure runs first. Lamp loom needs twenty color conductors plus suitably sized common return(s).</x:v>
+        <x:v>Use genuine rated parts with matching wire seals. Reused 14-pin machine connector excluded.</x:v>
       </x:c>
       <x:c r="K34" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=outdoor+multiconductor+copper+control+cable</x:v>
+        <x:v>https://www.amazon.com/s?k=Deutsch+DT+sealed+connector+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
@@ -1362,33 +1381,33 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
-        <x:v>Locking sealed cable connectors</x:v>
+        <x:v>Heat shrink, ferrules, loom and labels</x:v>
       </x:c>
       <x:c r="C35" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D35" s="3" t="str">
-        <x:v>set</x:v>
+        <x:v>small lot</x:v>
       </x:c>
       <x:c r="E35" s="12" t="n">
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F35" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G35" s="9" t="n">
         <x:f>C35*E35</x:f>
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
-        <x:v>Amazon / distributor</x:v>
+        <x:v>Amazon</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str"/>
       <x:c r="J35" s="24" t="str">
-        <x:v>Use genuine rated parts with matching wire seals. Reused 14-pin machine connector excluded.</x:v>
+        <x:v>Adhesive-lined shrink at splices; secure cable strain relief. Reduce if already owned.</x:v>
       </x:c>
       <x:c r="K35" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=Deutsch+DT+sealed+connector+kit</x:v>
+        <x:v>https://www.amazon.com/s?k=adhesive+lined+heat+shrink+ferrules+wire+labels</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
@@ -1396,7 +1415,7 @@
         <x:v>Assembly</x:v>
       </x:c>
       <x:c r="B36" s="22" t="str">
-        <x:v>Heat shrink, ferrules, loom and labels</x:v>
+        <x:v>Standoffs, fasteners and mounting brackets</x:v>
       </x:c>
       <x:c r="C36" s="21" t="n">
         <x:v>1</x:v>
@@ -1405,58 +1424,58 @@
         <x:v>small lot</x:v>
       </x:c>
       <x:c r="E36" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F36" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G36" s="23" t="n">
         <x:f>C36*E36</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H36" s="22" t="str">
-        <x:v>Amazon</x:v>
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str"/>
       <x:c r="J36" s="24" t="str">
-        <x:v>Adhesive-lined shrink at splices; secure cable strain relief. Reduce if already owned.</x:v>
+        <x:v>Insulated board clearance above steel plate; mounting should not puncture the sealing cavity.</x:v>
       </x:c>
       <x:c r="K36" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=adhesive+lined+heat+shrink+ferrules+wire+labels</x:v>
+        <x:v>https://www.amazon.com/s?k=nylon+pcb+standoff+M3+kit</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" s="3" t="str">
-        <x:v>Assembly</x:v>
+        <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
-        <x:v>Standoffs, fasteners and mounting brackets</x:v>
+        <x:v>Hammond 1554VA2GY opaque polycarbonate</x:v>
       </x:c>
       <x:c r="C37" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D37" s="3" t="str">
-        <x:v>small lot</x:v>
+        <x:v>box</x:v>
       </x:c>
       <x:c r="E37" s="12" t="n">
-        <x:v>7</x:v>
+        <x:v>43.5</x:v>
       </x:c>
       <x:c r="F37" s="3" t="str">
-        <x:v>Allowance</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="G37" s="9" t="n">
         <x:f>C37*E37</x:f>
-        <x:v>7</x:v>
+        <x:v>43.5</x:v>
       </x:c>
       <x:c r="H37" s="3" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str"/>
       <x:c r="J37" s="24" t="str">
-        <x:v>Insulated board clearance above steel plate; mounting should not puncture the sealing cavity.</x:v>
+        <x:v>Nominal 240 x 160 x 90 mm. Preferred planning size; confirm physical layout before drilling.</x:v>
       </x:c>
       <x:c r="K37" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=nylon+pcb+standoff+M3+kit</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/miniature_cases/1554va2gy</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
@@ -1464,33 +1483,33 @@
         <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B38" s="22" t="str">
-        <x:v>Hammond 1554VA2GY opaque polycarbonate</x:v>
+        <x:v>Hammond 1554VAPL mounting plate</x:v>
       </x:c>
       <x:c r="C38" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D38" s="22" t="str">
-        <x:v>box</x:v>
+        <x:v>plate</x:v>
       </x:c>
       <x:c r="E38" s="12" t="n">
-        <x:v>43.5</x:v>
+        <x:v>9.25</x:v>
       </x:c>
       <x:c r="F38" s="22" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G38" s="23" t="n">
         <x:f>C38*E38</x:f>
-        <x:v>43.5</x:v>
+        <x:v>9.25</x:v>
       </x:c>
       <x:c r="H38" s="22" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I38" s="3" t="str"/>
       <x:c r="J38" s="24" t="str">
-        <x:v>Nominal 240 x 160 x 90 mm. Preferred planning size; confirm physical layout before drilling.</x:v>
+        <x:v>Box plus plate clears advertised $49 free-shipping threshold; checkout confirmation still required.</x:v>
       </x:c>
       <x:c r="K38" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/miniature_cases/1554va2gy</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/subpanels/1554vapl</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
@@ -1498,33 +1517,33 @@
         <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B39" s="3" t="str">
-        <x:v>Hammond 1554VAPL mounting plate</x:v>
+        <x:v>Bimed BM-ENX-2S-W cable glands</x:v>
       </x:c>
       <x:c r="C39" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D39" s="3" t="str">
-        <x:v>plate</x:v>
+        <x:v>5-pack</x:v>
       </x:c>
       <x:c r="E39" s="12" t="n">
-        <x:v>9.25</x:v>
+        <x:v>3.25</x:v>
       </x:c>
       <x:c r="F39" s="3" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G39" s="9" t="n">
         <x:f>C39*E39</x:f>
-        <x:v>9.25</x:v>
+        <x:v>3.25</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str"/>
       <x:c r="J39" s="24" t="str">
-        <x:v>Box plus plate clears advertised $49 free-shipping threshold; checkout confirmation still required.</x:v>
+        <x:v>M12 x 1.5; jacket OD 3–6.5 mm. Use only where cable diameter fits; mounting hardware included.</x:v>
       </x:c>
       <x:c r="K39" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/enclosures_-a-_racks/subpanels/1554vapl</x:v>
+        <x:v>https://www.automationdirect.com/adc/shopping/catalog/wire_-a-_cable_management/cable_glands/metric_thread/bm-enx-2s-w</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
@@ -1532,33 +1551,33 @@
         <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B40" s="22" t="str">
-        <x:v>Bimed BM-ENX-2S-W cable glands</x:v>
+        <x:v>Larger glands, sealing plugs and seals</x:v>
       </x:c>
       <x:c r="C40" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D40" s="22" t="str">
-        <x:v>5-pack</x:v>
+        <x:v>allowance</x:v>
       </x:c>
       <x:c r="E40" s="12" t="n">
-        <x:v>3.25</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F40" s="22" t="str">
-        <x:v>Published</x:v>
+        <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G40" s="23" t="n">
         <x:f>C40*E40</x:f>
-        <x:v>3.25</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H40" s="22" t="str">
         <x:v>AutomationDirect</x:v>
       </x:c>
       <x:c r="I40" s="3" t="str"/>
       <x:c r="J40" s="24" t="str">
-        <x:v>M12 x 1.5; jacket OD 3–6.5 mm. Use only where cable diameter fits; mounting hardware included.</x:v>
+        <x:v>Machine/display cable may need larger glands or matched multi-hole inserts; measure first.</x:v>
       </x:c>
       <x:c r="K40" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/shopping/catalog/wire_-a-_cable_management/cable_glands/metric_thread/bm-enx-2s-w</x:v>
+        <x:v>https://www.automationdirect.com/adc/overview/catalog/wire_-a-_cable_management/cable_glands</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
@@ -1566,81 +1585,81 @@
         <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B41" s="3" t="str">
-        <x:v>Larger glands, sealing plugs and seals</x:v>
+        <x:v>Ten-lamp rail / rear wiring cover</x:v>
       </x:c>
       <x:c r="C41" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="3" t="str">
-        <x:v>allowance</x:v>
+        <x:v>assembly allowance</x:v>
       </x:c>
       <x:c r="E41" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F41" s="3" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G41" s="9" t="n">
         <x:f>C41*E41</x:f>
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H41" s="3" t="str">
-        <x:v>AutomationDirect</x:v>
+        <x:v>Local / Amazon</x:v>
       </x:c>
       <x:c r="I41" s="3" t="str"/>
       <x:c r="J41" s="24" t="str">
-        <x:v>Machine/display cable may need larger glands or matched multi-hole inserts; measure first.</x:v>
+        <x:v>Plan approximately 300 mm long; verify actual grommet diameter/pitch. No rated finished housing selected.</x:v>
       </x:c>
       <x:c r="K41" s="15" t="str">
-        <x:v>https://www.automationdirect.com/adc/overview/catalog/wire_-a-_cable_management/cable_glands</x:v>
+        <x:v>https://www.amazon.com/s?k=aluminum+u+channel+12+inch</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" s="22" t="str">
-        <x:v>Enclosure</x:v>
+        <x:v>Water</x:v>
       </x:c>
       <x:c r="B42" s="22" t="str">
-        <x:v>Ten-lamp rail / rear wiring cover</x:v>
+        <x:v>Manual shutoff and cleanable inlet strainer</x:v>
       </x:c>
       <x:c r="C42" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D42" s="22" t="str">
-        <x:v>assembly allowance</x:v>
+        <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E42" s="12" t="n">
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F42" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G42" s="23" t="n">
         <x:f>C42*E42</x:f>
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H42" s="22" t="str">
-        <x:v>Local / Amazon</x:v>
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I42" s="3" t="str"/>
       <x:c r="J42" s="24" t="str">
-        <x:v>Plan approximately 300 mm long; verify actual grommet diameter/pitch. No rated finished housing selected.</x:v>
+        <x:v>Reuse existing suitable items; select pressure rating and mesh for nozzle requirements.</x:v>
       </x:c>
       <x:c r="K42" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=aluminum+u+channel+12+inch</x:v>
+        <x:v>https://www.amazon.com/s?k=garden+hose+shut+off+valve+inline+filter+brass</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" s="3" t="str">
-        <x:v>Enclosure</x:v>
+        <x:v>Water</x:v>
       </x:c>
       <x:c r="B43" s="3" t="str">
-        <x:v>Meter electronics protection</x:v>
+        <x:v>Garden-hose to valve NPT fittings</x:v>
       </x:c>
       <x:c r="C43" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D43" s="3" t="str">
-        <x:v>assembly allowance</x:v>
+        <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E43" s="12" t="n">
         <x:v>15</x:v>
@@ -1653,14 +1672,14 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="H43" s="3" t="str">
-        <x:v>Local / distributor</x:v>
+        <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I43" s="3" t="str"/>
       <x:c r="J43" s="24" t="str">
-        <x:v>Dedicated splash/impact protection, supported plumbing and sealed terminations; exact housing pending geometry.</x:v>
+        <x:v>US garden hose thread is 3/4 GHT, distinct from 1/2 NPT valve threads. Include removable unions as required.</x:v>
       </x:c>
       <x:c r="K43" s="15" t="str">
-        <x:v>https://www.polycase.com/wp-series</x:v>
+        <x:v>https://www.amazon.com/s?k=3%2F4+GHT+to+1%2F2+NPT+brass+adapter</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
@@ -1668,47 +1687,47 @@
         <x:v>Water</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>Manual shutoff and cleanable inlet strainer</x:v>
+        <x:v>Straight pipe, washers, supports and sealant</x:v>
       </x:c>
       <x:c r="C44" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D44" s="22" t="str">
-        <x:v>set allowance</x:v>
+        <x:v>small lot</x:v>
       </x:c>
       <x:c r="E44" s="12" t="n">
-        <x:v>20</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F44" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G44" s="23" t="n">
         <x:f>C44*E44</x:f>
-        <x:v>20</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H44" s="22" t="str">
-        <x:v>Amazon / local</x:v>
+        <x:v>Local</x:v>
       </x:c>
       <x:c r="I44" s="3" t="str"/>
       <x:c r="J44" s="24" t="str">
-        <x:v>Reuse existing suitable items; select pressure rating and mesh for nozzle/meter requirements.</x:v>
+        <x:v>Choose supports and short pipe as the valve/hose layout requires; no meter-specific straight sections or NPS fittings.</x:v>
       </x:c>
       <x:c r="K44" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=garden+hose+shut+off+valve+inline+filter+brass</x:v>
+        <x:v>https://www.amazon.com/s?k=brass+1%2F2+NPT+pipe+nipple+plumbing</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" s="3" t="str">
-        <x:v>Water</x:v>
+        <x:v>Enclosure</x:v>
       </x:c>
       <x:c r="B45" s="3" t="str">
-        <x:v>Correct NPS meter adapters and seals</x:v>
+        <x:v>MG Chemicals 422C coating, small bottle</x:v>
       </x:c>
       <x:c r="C45" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D45" s="3" t="str">
-        <x:v>pair allowance</x:v>
+        <x:v>bottle allowance</x:v>
       </x:c>
       <x:c r="E45" s="12" t="n">
         <x:v>20</x:v>
@@ -1721,22 +1740,22 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="H45" s="3" t="str">
-        <x:v>Plumbing supplier</x:v>
+        <x:v>Amazon / distributor</x:v>
       </x:c>
       <x:c r="I45" s="3" t="str"/>
       <x:c r="J45" s="24" t="str">
-        <x:v>PROCUREMENT HOLD: straight NPS thread and actual seal geometry must match; NPT or cone-seat swivel is not assumed compatible.</x:v>
+        <x:v>Later, after testing; mask contacts, connectors and vents. Not a substitute for the gasketed box.</x:v>
       </x:c>
       <x:c r="K45" s="15" t="str">
-        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
+        <x:v>https://www.amazon.com/s?k=MG+Chemicals+422C+55ml</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" s="22" t="str">
-        <x:v>Water</x:v>
+        <x:v>Bench</x:v>
       </x:c>
       <x:c r="B46" s="22" t="str">
-        <x:v>Garden-hose to valve NPT fittings</x:v>
+        <x:v>Temporary fused battery lead and small fuses</x:v>
       </x:c>
       <x:c r="C46" s="21" t="n">
         <x:v>1</x:v>
@@ -1745,195 +1764,141 @@
         <x:v>set allowance</x:v>
       </x:c>
       <x:c r="E46" s="12" t="n">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F46" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G46" s="23" t="n">
         <x:f>C46*E46</x:f>
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H46" s="22" t="str">
         <x:v>Amazon / local</x:v>
       </x:c>
       <x:c r="I46" s="3" t="str"/>
       <x:c r="J46" s="24" t="str">
-        <x:v>US garden hose thread is 3/4 GHT, distinct from 1/2 NPT valve threads. Include removable unions as required.</x:v>
+        <x:v>Bench only, close to battery; size fuse to test stage and weakest wire. Not a new machine fuse block.</x:v>
       </x:c>
       <x:c r="K46" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=3%2F4+GHT+to+1%2F2+NPT+brass+adapter</x:v>
+        <x:v>https://www.amazon.com/s?k=inline+ATO+fuse+holder+1A+2A+fuse</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" s="3" t="str">
-        <x:v>Water</x:v>
+        <x:v>Bench</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>Straight pipe, washers, supports and sealant</x:v>
+        <x:v>250-ohm 0.1% 0.5 W removable test resistor</x:v>
       </x:c>
       <x:c r="C47" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D47" s="3" t="str">
-        <x:v>small lot</x:v>
+        <x:v>resistor allowance</x:v>
       </x:c>
       <x:c r="E47" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>3.36</x:v>
       </x:c>
       <x:c r="F47" s="3" t="str">
-        <x:v>Allowance</x:v>
+        <x:v>Published</x:v>
       </x:c>
       <x:c r="G47" s="9" t="n">
         <x:f>C47*E47</x:f>
-        <x:v>8</x:v>
+        <x:v>3.36</x:v>
       </x:c>
       <x:c r="H47" s="3" t="str">
-        <x:v>Local</x:v>
+        <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I47" s="3" t="str"/>
       <x:c r="J47" s="24" t="str">
-        <x:v>Respect meter straight lengths and seal type. Do not seal NPS solely with PTFE tape.</x:v>
+        <x:v>Vishay RN65E2500BB14: 250 ohm, 0.1%, 0.5 W. Removable DAC bench load only; never add as a permanent valve/feedback shunt.</x:v>
       </x:c>
       <x:c r="K47" s="15" t="str">
-        <x:v>https://www.sciosense.com/ufm-02-ultrasonic-flow-sensing-module/</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/vishay-dale/RN65E2500BB14/3193953</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" s="22" t="str">
-        <x:v>Enclosure</x:v>
+        <x:v>Bench</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>MG Chemicals 422C coating, small bottle</x:v>
+        <x:v>Micro-USB data cable</x:v>
       </x:c>
       <x:c r="C48" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D48" s="22" t="str">
-        <x:v>bottle allowance</x:v>
+        <x:v>cable allowance</x:v>
       </x:c>
       <x:c r="E48" s="12" t="n">
-        <x:v>20</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F48" s="22" t="str">
         <x:v>Allowance</x:v>
       </x:c>
       <x:c r="G48" s="23" t="n">
         <x:f>C48*E48</x:f>
-        <x:v>20</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H48" s="22" t="str">
-        <x:v>Amazon / distributor</x:v>
+        <x:v>Amazon / existing</x:v>
       </x:c>
       <x:c r="I48" s="3" t="str"/>
       <x:c r="J48" s="24" t="str">
-        <x:v>Later, after testing; mask contacts, connectors and vents. Not a substitute for the gasketed box.</x:v>
+        <x:v>Set quantity to zero if owned. Must carry data, not charging-only.</x:v>
       </x:c>
       <x:c r="K48" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=MG+Chemicals+422C+55ml</x:v>
+        <x:v>https://www.amazon.com/s?k=micro+usb+data+cable</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
-      <x:c r="A49" s="3" t="str">
-        <x:v>Bench</x:v>
-      </x:c>
-      <x:c r="B49" s="3" t="str">
-        <x:v>Temporary fused battery lead and small fuses</x:v>
-      </x:c>
-      <x:c r="C49" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D49" s="3" t="str">
-        <x:v>set allowance</x:v>
-      </x:c>
-      <x:c r="E49" s="12" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F49" s="3" t="str">
-        <x:v>Allowance</x:v>
-      </x:c>
+      <x:c r="A49" s="3"/>
+      <x:c r="B49" s="3"/>
+      <x:c r="C49" s="21"/>
+      <x:c r="D49" s="3"/>
+      <x:c r="E49" s="12"/>
+      <x:c r="F49" s="3"/>
       <x:c r="G49" s="9" t="n">
         <x:f>C49*E49</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="H49" s="3" t="str">
-        <x:v>Amazon / local</x:v>
-      </x:c>
-      <x:c r="I49" s="3" t="str"/>
-      <x:c r="J49" s="24" t="str">
-        <x:v>Bench only, close to battery; size fuse to test stage and weakest wire. Not a new machine fuse block.</x:v>
-      </x:c>
-      <x:c r="K49" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=inline+ATO+fuse+holder+1A+2A+fuse</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H49" s="3"/>
+      <x:c r="I49" s="3"/>
+      <x:c r="J49" s="24"/>
+      <x:c r="K49" s="15"/>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
-      <x:c r="A50" s="22" t="str">
-        <x:v>Bench</x:v>
-      </x:c>
-      <x:c r="B50" s="22" t="str">
-        <x:v>250-ohm 0.1% 0.5 W removable test resistor</x:v>
-      </x:c>
-      <x:c r="C50" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D50" s="22" t="str">
-        <x:v>resistor allowance</x:v>
-      </x:c>
-      <x:c r="E50" s="12" t="n">
-        <x:v>3.36</x:v>
-      </x:c>
-      <x:c r="F50" s="22" t="str">
-        <x:v>Published</x:v>
-      </x:c>
+      <x:c r="A50" s="22"/>
+      <x:c r="B50" s="22"/>
+      <x:c r="C50" s="21"/>
+      <x:c r="D50" s="22"/>
+      <x:c r="E50" s="12"/>
+      <x:c r="F50" s="22"/>
       <x:c r="G50" s="23" t="n">
         <x:f>C50*E50</x:f>
-        <x:v>3.36</x:v>
-      </x:c>
-      <x:c r="H50" s="22" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I50" s="3" t="str"/>
-      <x:c r="J50" s="24" t="str">
-        <x:v>Vishay RN65E2500BB14: 250 ohm, 0.1%, 0.5 W. Removable DAC bench load only; never add as a permanent valve/feedback shunt.</x:v>
-      </x:c>
-      <x:c r="K50" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/vishay-dale/RN65E2500BB14/3193953</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H50" s="22"/>
+      <x:c r="I50" s="3"/>
+      <x:c r="J50" s="24"/>
+      <x:c r="K50" s="15"/>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
-      <x:c r="A51" s="3" t="str">
-        <x:v>Bench</x:v>
-      </x:c>
-      <x:c r="B51" s="3" t="str">
-        <x:v>Micro-USB data cable</x:v>
-      </x:c>
-      <x:c r="C51" s="21" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D51" s="3" t="str">
-        <x:v>cable allowance</x:v>
-      </x:c>
-      <x:c r="E51" s="12" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F51" s="3" t="str">
-        <x:v>Allowance</x:v>
-      </x:c>
+      <x:c r="A51" s="3"/>
+      <x:c r="B51" s="3"/>
+      <x:c r="C51" s="21"/>
+      <x:c r="D51" s="3"/>
+      <x:c r="E51" s="12"/>
+      <x:c r="F51" s="3"/>
       <x:c r="G51" s="9" t="n">
         <x:f>C51*E51</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H51" s="3" t="str">
-        <x:v>Amazon / existing</x:v>
-      </x:c>
-      <x:c r="I51" s="3" t="str"/>
-      <x:c r="J51" s="24" t="str">
-        <x:v>Set quantity to zero if owned. Must carry data, not charging-only.</x:v>
-      </x:c>
-      <x:c r="K51" s="15" t="str">
-        <x:v>https://www.amazon.com/s?k=micro+usb+data+cable</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H51" s="3"/>
+      <x:c r="I51" s="3"/>
+      <x:c r="J51" s="24"/>
+      <x:c r="K51" s="15"/>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" s="3"/>
@@ -2084,7 +2049,7 @@
       <x:c r="H60" s="3"/>
       <x:c r="I60" s="3"/>
       <x:c r="J60" s="24" t="str">
-        <x:v>Combined allowance for two supplier baskets; neither is a destination quote</x:v>
+        <x:v>Combined allowance for DigiKey passives/regulator and Mouser relay; neither is a destination quote</x:v>
       </x:c>
       <x:c r="K60" s="15" t="str">
         <x:v>https://www.mouser.com/en/ProductDetail/Panasonic-Industry/TQ2-5V?qs=HLLy2pIPwutHaTSpVfb1kw%3D%3D</x:v>
@@ -2175,7 +2140,7 @@
     </x:row>
     <x:row r="66" ht="26" customHeight="1">
       <x:c r="A66" s="20" t="str">
-        <x:v>Installed quantities match Rev D. Reused X1 costs $0. The separate 250-ohm test resistor is on row 50.</x:v>
+        <x:v>Installed quantities match Rev E. Reused X1 costs $0. The separate 250-ohm test resistor is in the main basket.</x:v>
       </x:c>
       <x:c r="B66" s="20"/>
       <x:c r="C66" s="20"/>
@@ -2223,7 +2188,7 @@
     </x:row>
     <x:row r="68" ht="66" customHeight="1">
       <x:c r="A68" s="24" t="str">
-        <x:v>R1, R2, R3, R4, R8, R9</x:v>
+        <x:v>R1, R2, R3, R4</x:v>
       </x:c>
       <x:c r="B68" s="24" t="str">
         <x:v>MFR-50FTE52-1K</x:v>
@@ -2232,7 +2197,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D68" s="31" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E68" s="30" t="n">
         <x:v>0.076</x:v>
@@ -2291,173 +2256,152 @@
     </x:row>
     <x:row r="70" ht="66" customHeight="1">
       <x:c r="A70" s="24" t="str">
-        <x:v>R6, R7</x:v>
+        <x:v>D1, D2, D3, D4</x:v>
       </x:c>
       <x:c r="B70" s="24" t="str">
-        <x:v>MFR-25FBF52-4K7</x:v>
+        <x:v>1N4148 (onsemi)</x:v>
       </x:c>
       <x:c r="C70" s="25" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="D70" s="31" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E70" s="30" t="n">
-        <x:v>0.044</x:v>
+        <x:v>0.06</x:v>
       </x:c>
       <x:c r="F70" s="24" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G70" s="27" t="n">
         <x:f>C70*E70</x:f>
-        <x:v>0.43999999999999995</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H70" s="24" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I70" s="24" t="str"/>
       <x:c r="J70" s="24" t="str">
-        <x:v>4.7 kohm, 1%, 0.25 W axial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+        <x:v>1N4148 axial DO-35; band = cathode; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
       </x:c>
       <x:c r="K70" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-4K7/9138176</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/onsemi/1N4148/458603</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="66" customHeight="1">
       <x:c r="A71" s="28" t="str">
-        <x:v>D1, D2, D3, D4</x:v>
+        <x:v>C1, C5, C10, C11, C12</x:v>
       </x:c>
       <x:c r="B71" s="28" t="str">
-        <x:v>1N4148 (onsemi)</x:v>
+        <x:v>C315C104K5R5TA</x:v>
       </x:c>
       <x:c r="C71" s="25" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="D71" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E71" s="30" t="n">
-        <x:v>0.06</x:v>
+        <x:v>0.488</x:v>
       </x:c>
       <x:c r="F71" s="28" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G71" s="29" t="n">
         <x:f>C71*E71</x:f>
-        <x:v>0.6</x:v>
+        <x:v>4.88</x:v>
       </x:c>
       <x:c r="H71" s="28" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I71" s="24" t="str"/>
       <x:c r="J71" s="24" t="str">
-        <x:v>1N4148 axial DO-35; band = cathode; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+        <x:v>100 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
       </x:c>
       <x:c r="K71" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/onsemi/1N4148/458603</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/kemet/C315C104K5R5TA/12701330</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="66" customHeight="1">
       <x:c r="A72" s="24" t="str">
-        <x:v>C1, C2, C5, C10, C11, C12</x:v>
+        <x:v>C4</x:v>
       </x:c>
       <x:c r="B72" s="24" t="str">
-        <x:v>C315C104K5R5TA</x:v>
+        <x:v>SR305C334KARTR1</x:v>
       </x:c>
       <x:c r="C72" s="25" t="n">
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D72" s="31" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E72" s="30" t="n">
-        <x:v>0.488</x:v>
+        <x:v>1.48</x:v>
       </x:c>
       <x:c r="F72" s="24" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G72" s="27" t="n">
         <x:f>C72*E72</x:f>
-        <x:v>4.88</x:v>
+        <x:v>2.96</x:v>
       </x:c>
       <x:c r="H72" s="24" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I72" s="24" t="str"/>
       <x:c r="J72" s="24" t="str">
-        <x:v>100 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+        <x:v>330 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
       </x:c>
       <x:c r="K72" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/kemet/C315C104K5R5TA/12701330</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/kyocera-avx/SR305C334KARTR1/9948632</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="66" customHeight="1">
       <x:c r="A73" s="28" t="str">
-        <x:v>C4</x:v>
+        <x:v>C7, C8, C9</x:v>
       </x:c>
       <x:c r="B73" s="28" t="str">
-        <x:v>SR305C334KARTR1</x:v>
+        <x:v>EEU-FC1V470B</x:v>
       </x:c>
       <x:c r="C73" s="25" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D73" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E73" s="30" t="n">
-        <x:v>1.48</x:v>
+        <x:v>0.48</x:v>
       </x:c>
       <x:c r="F73" s="28" t="str">
         <x:v>Published</x:v>
       </x:c>
       <x:c r="G73" s="29" t="n">
         <x:f>C73*E73</x:f>
-        <x:v>2.96</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="H73" s="28" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I73" s="24" t="str"/>
       <x:c r="J73" s="24" t="str">
-        <x:v>330 nF, 50 V, X7R, radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
+        <x:v>47 uF, 35 V, 105 C, polarized radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
       </x:c>
       <x:c r="K73" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/kyocera-avx/SR305C334KARTR1/9948632</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/panasonic-industry/EEU-FC1V470B/16639056</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="66" customHeight="1">
-      <x:c r="A74" s="24" t="str">
-        <x:v>C7, C8, C9</x:v>
-      </x:c>
-      <x:c r="B74" s="24" t="str">
-        <x:v>EEU-FC1V470B</x:v>
-      </x:c>
-      <x:c r="C74" s="25" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D74" s="31" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E74" s="30" t="n">
-        <x:v>0.48</x:v>
-      </x:c>
-      <x:c r="F74" s="24" t="str">
-        <x:v>Published</x:v>
-      </x:c>
-      <x:c r="G74" s="27" t="n">
-        <x:f>C74*E74</x:f>
-        <x:v>2.4</x:v>
-      </x:c>
-      <x:c r="H74" s="24" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I74" s="24" t="str"/>
-      <x:c r="J74" s="24" t="str">
-        <x:v>47 uF, 35 V, 105 C, polarized radial; observed small-quantity / cut-tape price, 7 Oct 2026.</x:v>
-      </x:c>
-      <x:c r="K74" s="15" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/panasonic-industry/EEU-FC1V470B/16639056</x:v>
-      </x:c>
+      <x:c r="A74" s="24"/>
+      <x:c r="B74" s="24"/>
+      <x:c r="C74" s="25"/>
+      <x:c r="D74" s="31"/>
+      <x:c r="E74" s="30"/>
+      <x:c r="F74" s="24"/>
+      <x:c r="G74" s="27"/>
+      <x:c r="H74" s="24"/>
+      <x:c r="I74" s="24"/>
+      <x:c r="J74" s="24"/>
+      <x:c r="K74" s="15"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="18" t="str"/>
@@ -2470,12 +2414,12 @@
       </x:c>
       <x:c r="G75" s="33" t="n">
         <x:f>SUM(G68:G74)</x:f>
-        <x:v>12.459999999999999</x:v>
+        <x:v>12.020000000000001</x:v>
       </x:c>
       <x:c r="H75" s="18" t="str"/>
       <x:c r="I75" s="3" t="str"/>
       <x:c r="J75" s="3" t="str">
-        <x:v>Included once through E30. No extra fee or shipping added here.</x:v>
+        <x:v>Included once through E29. No extra fee or shipping added here.</x:v>
       </x:c>
       <x:c r="K75" s="3" t="str"/>
     </x:row>

</xml_diff>